<commit_message>
daily: 2026-09-14 日報 HTML & Excel 更新
由 2026-09-15 排程補提交：9/14 的報表與 Excel 已於當日產出，惟未執行 commit。

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -895,7 +895,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-09-11</t>
+          <t>報告更新日期：2026-09-14</t>
         </is>
       </c>
     </row>
@@ -3333,7 +3333,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G124"/>
+  <dimension ref="A1:G125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3355,7 +3355,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-09-11</t>
+          <t>最後更新：2026-09-14</t>
         </is>
       </c>
     </row>
@@ -7898,6 +7898,60 @@
         </is>
       </c>
     </row>
+    <row r="125">
+      <c r="A125" s="50" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B125" s="50" t="inlineStr">
+        <is>
+          <t>NT$2,410（9/11收）</t>
+        </is>
+      </c>
+      <c r="C125" s="57" t="inlineStr">
+        <is>
+          <t>-1.63%（9/11收）</t>
+        </is>
+      </c>
+      <c r="D125" s="50" t="inlineStr">
+        <is>
+          <t>US$433.24（9/11收）</t>
+        </is>
+      </c>
+      <c r="E125" s="50" t="inlineStr">
+        <is>
+          <t>21,131（9/11收）</t>
+        </is>
+      </c>
+      <c r="F125" s="52" t="inlineStr">
+        <is>
+          <t>報告日2026-09-14(Mon)，台股資料為2026-09-11(Fri)官方收盤；ADR、費半與全部美股個股為9/11美東收盤(台北9/12清晨)。9/12至9/13為週末，無交易資料。
+(1)⚠️⚠️本報今日的內容分成方向完全相反的兩段，必須兩段合看才不會誤判，這是本日最重要的一件事。第一段是9/11台股收盤的四項轉弱證據；第二段是台股收盤「之後」才發生的美股反彈與今晨夜盤大漲。今日日報所依據的最新收盤是在利多發生之前形成的——技術面的轉弱確認是事實，但它描述的是上週五收盤當下的狀態，不是今日開盤後的狀態。本報依約將立場自「中性」下修為「中性偏空」(下修半級而非依前報字面直接轉為偏空，理由即為證據的時序)。
+(2)台股2330官方收NT$2,410(-40、-1.63%、開2,430／高2,430／低2,405、量21,131張、額NT$510.50億、164,402筆，TWSE STOCK_DAY確認)，連3日收黑且跌幅逐日擴大(-0.20%→-0.61%→-1.63%)。⚠️⚠️型態是本波最弱的一根K線：開盤2,430即為全日最高，全場未能再觸及開盤價(本報追蹤期間首見)，收盤距最低點僅5點，無上影線。⚠️本報必須撤回前一日對9/10那根下影線的樂觀解讀：9/10記錄「2,435至2,440一帶出現實質承接」，9/11該承接在一天內即被穿透，最低價下移30點至2,405。⭐惟本報9/10已寫明「下影線只證明有買盤、不證明買盤能推動價格」，該保留在隔日即獲驗證。高點連續第4個交易日降低(2,505→2,490→2,455→2,430)。筆數164,402較9/10的85,691近乎倍增(+91.9%)，平均每筆僅0.13張，屬散戶承接放大特徵。
+(3)⭐前報所訂檢核價位的答案須誠實處理、不取巧：前報訂下「具體檢核價位為20日均線暨布林中軌2,410：今日若收在其下，須再下修至偏空」。9/11實際收盤恰好是2,410——字面上「收在其下」不成立(收盤等於該價位、並非低於)。⚠️⚠️但本報不採用這個對自己有利的讀法：前報寫下2,410時用的是9/10當日的20日均線值，而9/11當日的20日均線已上移至2,411，以當日中軌計算收盤實際低於中軌1點。本報的處理是兩種讀法並陳並取其實質：跌破成立，但幅度僅1點(0.04%)，與9/10跌破5日均線時的量級完全相同，屬「貼線」而非「破線」。
+(4)⚠️⚠️前報所訂的兩項轉弱確認條件則毫無模糊空間、雙雙成立：(a)KDJ——前報原話「J值64.32距50尚有14.32點，若J跌破50且D開始下彎，才構成中期轉弱確認」，9/11的J重挫32.49點至31.83、低於50達18.17點，D自68.13降至62.94確實轉為下彎，兩項條件均成立；K自66.86降至52.57，與D的負乖離自1.27點擴大至10.37點(8.2倍)。⚠️惟須並陳一項保留：J值31.83已接近一般視為短線超賣的20至30區間，「轉弱確認」與「短線超賣」在本日同時成立、方向相反。(b)均線——前報原話「若連續兩日收在MA5之下，均線結構才會進入實質轉弱」，9/10收2,450、9/11收2,410連續兩日成立，距離自1點擴大至41點。本日並新增跌破MA10(2,429)與MA20(2,411)，五線失守三線，僅餘MA60(2,400)與MA120(2,277)；短均已轉向(MA10自2,430降至2,429)、中長均線尚未(MA20、MA60、MA120仍上彎)。
+(5)⚠️其餘技術指標同步轉弱：RSI(14)自55.83重挫5.81點至50.02，連3日下滑且本日跌幅為三日中最大(-0.79、-2.35、-5.81)，恰停在多空分界線上方0.02點。⭐MACD紅柱自+11.04急縮至+3.96(-64.1%)，為四項中唯一正值；拆解成因：DIF自19.33降至16.29(下彎)、DEA自13.81升至14.31(仍上行)，兩線差距僅剩1.98點，為死叉形成前的標準型態。布林通道2,474／2,411／2,348，收盤2,410位於中軌之下1點。5日均量22,919張，9/11量21,131張低於均量7.8%，連3日未站回均量。⭐技術指標口徑驗證：以同一套算法回算9/10已發布值(RSI 55.83／MACD柱11.04／K 66.86／D 68.13／J 64.32／MA5 2,451／MA10 2,430／MA20 2,410／MA60 2,399／MA120 2,272／布林2,474-2,410-2,347／5日均量21,513)全數完全複現，確認口徑未漂移。
+(6)⚠️⚠️籌碼面是本日最硬的偏空證據，規模而非方向才是重點：外資9/11賣超8,251張(TWSE T86官方-8,251,130股)，為本報追蹤期間單日最大賣超，規模較9/10的-1,944張擴大4.24倍，連續第3日賣超；投信賣超181張(連3日賣超但規模收斂59.6%)；自營商賣超400張(自行買賣-544,700股→-545張、避險+144,239股→+144張)。三大法人分項加總合計賣超8,832張，與官方合計欄位(-8,832,445股)換算值完全一致。⭐緩解證據有二且不宜誇大：近5日(9/7至9/11)外資合計仍淨買超8,878張(+16,135、+5,497、-2,559、-1,944、-8,251)，連3日賣超12,754張已回吐9/7單日買超16,135張的79.0%；⚠️但這個緩衝已經薄了——再一個同等規模的賣超日就會把5日合計翻負，本報認為這是今日最值得追蹤的單一數字。
+(7)⭐期貨端方向與現貨相反，是本日少數偏多的籌碼證據：CDF 202609日盤收2,418(-29、-1.19%、成交9,542口、結算價2,416)，基差自-2點翻回+8點正價差——現貨大跌1.63%的一天期貨相對抗跌。未平倉自18,850口降至15,320口(-3,530口)，⚠️但本報自本日起不再把它單獨解讀為「部位撤出」：9/16為9月月結算日，轉倉已啟動，同日CDF 202610未平倉已達12,820口，兩者合計28,140口反而高於9/10的近月單一水位。台指期TX 202609日盤收46,218(-651、成交58,137口、未平倉88,464口)。三大法人台指期部位：外資淨空單85,067口、投信淨多單74,687口、自營淨多單2,802口(⚠️此為大盤層級部位，不可直接讀為對台積電個股的看法)。
+(8)⚠️TXO的P/C未平倉比0.88(賣權52,641口／買權60,025口、官方比率欄87.70%)。⚠️9/11(週五)為TXO到期結算日，雙邊未平倉大幅結清重建(賣權69,363→52,641口、買權83,906→60,025口，雙邊自153,269口降至112,666口、-26.5%)，比率的變化幅度不具參考價值，只能看絕對水位。⭐絕對水位本身是少數偏多訊號：0.88明顯低於1(買權未平倉多出7,384口、14.0%)，依本報既定分段屬「中性偏多」。⚠️三項保留：結算後為全新基期、只有次一交易日起的變化才有意義；本週三9/16為月結算日將再次重置，故本週實際上只有週一(9/14)與週二(9/15)兩天具備跨日可比性；此為台指選擇權(大盤)非台積電個股數據。
+(9)⭐⭐第二段：台股收盤之後方向完全相反。美國8月CPI於美東9/11上午8:30公布，核心年增2.4%為2021年3月以來最低(整體3.4%、與7月持平、月增0.4%，核心月增0.3%高於市場預期0.2%，來源：BLS官方／CNBC經Yahoo Finance轉載)。美股四大指數全面反彈：標普+0.86%收7,656.98、那斯達克+0.96%收26,333.04、道瓊+0.98%收52,573.29、VIX自17.84降至15.84(-11.2%)。⭐費半+1.81%收11,824.00領漲大盤，終結9/10的-2.66%(追蹤區間最大單日跌幅)，惟僅收復其約三分之二。ADR收$433.24(+5.21、+1.22%)。⚠️兩項保留必須並陳：(a)核心月增0.3%高於預期，10年期公債殖利率不降反升至4.97%(前一日4.94%)——市場買的是「核心年增創四年半新低」這半邊，對利率路徑的疑慮並未解除；(b)費半的反彈並非由龍頭領導——輝達收$218.29(-0.03%)連4日收黑、美光-0.22%連2日收黑，兩者是族群反彈日中僅有的收黑者，領漲的是前一日跌最重的Amkor(+4.44%)、Arm(+4.17%)、高通(+2.88%、連4紅創本波新高)、英特爾(+2.61%)、超微(+2.49%)——這種結構比較像超跌反彈而非趨勢重啟。⚠️本報另須標明一項未能證實：多則次級來源稱CPI後市場對9月FOMC的討論集中在「升息」而非降息(機率約65%、另有85.5%之說)，惟未能於BLS、CNBC、Reuters一手原文核實該機率數字，故僅轉述不採信。
+(10)⭐今晨夜盤已先行給出方向，為今日唯一可用於推估開盤的即時證據：TAIFEX日期標記9/14的「盤後」列(即9/11 15:00至今晨05:00那一段)，台指期202609收46,588(+401、開46,306／高46,663／低46,041、量28,667口)，台積電個股期CDF 202609收2,434(+18、開2,423／高2,442／低2,414、量1,520口)——CDF夜盤收盤較9/11現貨收盤2,410高出24點(+1.00%)，指向今日開高。⚠️三項保留：夜盤量僅1,520口為日盤9,542口的15.9%、代表性有限；夜盤價不是收盤價，開高後能否守住才是重點；前一份日報的相同欄位曾預告「今晨夜盤CDF重挫32點至2,415」而當日收盤2,410確實低於該夜盤價5點——夜盤方向對了但幅度會被日盤修正，這次的+24點同樣不應被當成當日漲幅的預測值。
+(11)⚠️⚠️9/11的亞洲時段與美國時段方向完全相反，這是最容易被忽略卻最該記錄的結構性觀察：亞洲時段——台股加權指數收46,184.85(-755.64點、-1.61%，為本報追蹤期間最大單日跌點)，台積電-1.63%、日月光-4.92%(收618.00元、回吐連2日逆勢漲幅、為全部追蹤標的中當日跌幅最大)、華邦電-4.46%(171.50元)、聯發科-2.86%(4,585元)；韓股三星電子-3.53%收259,500韓元、SK海力士-2.21%收1,812,000韓元(⚠️韓股採9/11收盤日線，未採Yahoo meta，因本報產製時韓股9/14已開盤、meta為盤中價)。美股時段——費半+1.81%、ADR+1.22%。⭐判讀兩層：亞洲時段的下跌發生在CPI公布之前，屬對9/10美股重挫的遞延反應而非對新資訊的反應；且台積電-1.63%在台股半導體族群中反而是相對抗跌的一檔——本報9/10記錄的「台積電連兩日為族群內相對弱勢股」在9/11已經逆轉。
+(12)⭐評價：TWSE官方BWIBBU 9/11顯示P/E 27.94x、P/B 9.72x、殖利率0.91%(9/10為28.40x／9.88x／0.90%)，財報基準維持115/2未變動。⭐算術自我檢核兩道：P/E降幅-1.62%、P/B降幅-1.62%，與股價跌幅-1.63%一致(差異僅來自四捨五入)，確認分母未動、純為股價效果；以每股淨值248.05直接驗算2,410÷248.05＝9.716≈9.72，與官方值相符。市值約NT$62.5兆。ADR端P/E約31.8x、P/B約11.1x，係依官方值×(1+溢價13.72%)換算。⚠️百分位欄位(5年88%／10年89%／P/B 92%)為8/14換基準時的粗略重校值，本報並未每日重算。
+(13)⭐ADR溢價自10.24%大幅擴大至13.72%(+3.48個百分點)，但成因幾乎全部是時間差、不是評價差：理論平價＝5×2,410÷31.63＝380.97(採捨入後匯率)，對市價433.24之溢價+13.72%。⚠️台股9/11收盤在台北13:30、ADR 9/11收盤在台北9/12清晨04:00，中間隔了CPI公布與美股反彈——溢價擴大代表的是「台股尚未反映美股的反彈」，而非外資對台積電更樂觀。⭐可操作意義：13.72%落在本報近月觀察區間(約9至14%)的上緣，兩地價差偏大、易向下收斂；⚠️惟收斂可由台股補漲達成、也可由ADR回跌達成，本報無法判定何者，不做方向性推論。⭐相對強弱：台積電-1.63%與加權指數-1.61%幾乎同幅(僅落後0.02個百分點)——本日台積電並未較大盤弱，弱的是整個台股。期間比較：近5日+0.00%(基準9/4收2,410，本波自9/4起的漲勢至9/11已全數回吐、五日報酬歸零)，大盤近5日-0.79%已轉負，台積電反而相對抗跌；近1月+0.63%(基準日曆同日減一月為8/11收2,395，⚠️基準自前一版的8/10之2,380上移15點，本欄的下降有一部分來自滾動窗口的機械效果)，大盤+2.36%；YTD+52.1%(基準2026-01-02收1,585)，落後大盤+57.4%與費半+60.5%。
+(14)⚠️匯率連2日走貶：新台幣9/11 16:00台北時點報31.634(本報採31.63)，較9/10的31.547再貶0.28%，⭐方向對台積電以美元計價的營收換算有利。⚠️取數限制須標明：Yahoo TWD=X的9/11日線K棒缺漏——判定為Yahoo序列自身缺漏而非台灣休市(同日2330.TW與韓股均有K棒)，本報改採同一來源的小時線、取台北9/11 16:00讀數，非內插、非以盤中價冒充收盤。
+(15)⚠️⚠️本週三9/16(僅剩2個交易日)將有兩個技術性事件同日發生，性質互不相關但極易互相污染判讀，本報提前提醒：(a)台股2330除息，每股現金股利NT$7.00001(TWSE官方除權除息預告表TWT48U，本日以查詢區間2026-09-01至10-31第三度查得，2330為該區間68筆之一，申報基準115年第2季、每股淨值248.05、每股盈餘49.33，三日數字完全一致)；以9/11收盤2,410計除息參考價約2,403，股價機械性扣除約7點(-0.29%)，P/E與P/B同步機械性下降——讀者在比較9/16之後的股價時務必還原此缺口，勿把除息誤讀為下跌。(b)9/16為2026年9月的第三個週三，即台指期貨與選擇權的月結算日；選擇權未平倉將大幅結清重建，台指期與台積電個股期換月至202610合約，未平倉躍升屬轉倉而非新增部位，且新舊合約的收盤價、結算價與價差不可跨合約比較。⚠️兩者疊加後，9/16當日的價格、量能、未平倉與P/C比四項數據會被兩種技術性因素同時干擾，本報屆時將逐項區分。⭐ADR股利金額維持9/11版結論：NT$7.00001×5÷匯率約31.42≈US$1.114，與CNBC所載一致；⚠️台積電IR官網(investor.tsmc.com)持續回HTTP 403、未能取得一手公告，故ADR金額標示為【以台股股利換算，待官方確認】。12/10為8/11董事會核准之Q2 2026股利(NT$7.0/股、基準日12/16)除息日，與9/16屬不同批次。
+(16)⭐產業消息：TrendForce於9/11報導，三星晶圓代工2nm GAA製程良率已自年初的不到50%提升至逾70%，製程漸趨穩定；但與高通的2nm合作因價格談判膠著，量產時程恐自2026年底延後至2027年；三星德州Taylor廠2nm產能已被特斯拉、博通、Arm訂單預先訂滿。⚠️判讀須分兩層：良率突破70%是中長期競爭威脅；⭐但高通這個指標性客戶的訂單延宕，短期反而降低台積電N2客戶流失的近期風險，而台積電N2已於9/9隨iPhone 18 Pro的A20 Pro進入實際量產出貨。⭐蘋果9/11收$332.27(+1.75%)連2日收紅再創本波新高，兩日自$315.34累計+5.4%；⚠️本報9/11版曾記錄「未能取得蘋果9/10當日的明確個股觸發新聞」，本次查證同樣未能取得9/11的個股觸發新聞，僅記錄事實、不對漲因下定論。⚠️本次查證未發現台積電官網(pr.tsmc.com)於9/10之後有任何新發布的新聞稿，9/11至9/14窗口內台積電本身無新公告。
+(17)⭐⭐今日第一順位觀察非常明確：夜盤指向開高，關鍵不在能否開高，而在開高後能否收復20日均線2,411與10日均線2,429——收復即可將上週五的跌破確認為假跌破，未能收復則本報將在明日進一步下修。第二順位為外資是否隨美股反彈轉為買超(若再現同等規模賣超日，5日合計翻負，須再下修至偏空)。第三順位為60MA季線2,400，它是目前唯一尚未被測試的支撐，距9/11收盤僅10點。</t>
+        </is>
+      </c>
+      <c r="G125" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:G2"/>

</xml_diff>

<commit_message>
daily: 2026-09-15 日報 HTML & Excel 更新
台股 9/14 收 2,380（-1.24%），跌破 60MA 季線，四項技術指標同日全轉空；
外資賣超 11,191 張。台股收盤後美股半導體崩跌（費半 -5.86%、ADR -3.52%），
尚未反映於台股。立場自中性偏空下修為看空。

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -895,7 +895,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-09-14</t>
+          <t>報告更新日期：2026-09-15</t>
         </is>
       </c>
     </row>
@@ -3333,7 +3333,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G125"/>
+  <dimension ref="A1:G126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3355,7 +3355,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-09-14</t>
+          <t>最後更新：2026-09-15</t>
         </is>
       </c>
     </row>
@@ -7952,6 +7952,60 @@
         </is>
       </c>
     </row>
+    <row r="126">
+      <c r="A126" s="53" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B126" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,380（9/14收）</t>
+        </is>
+      </c>
+      <c r="C126" s="56" t="inlineStr">
+        <is>
+          <t>-1.24%（9/14收）</t>
+        </is>
+      </c>
+      <c r="D126" s="53" t="inlineStr">
+        <is>
+          <t>US$418.01（9/14收）</t>
+        </is>
+      </c>
+      <c r="E126" s="53" t="inlineStr">
+        <is>
+          <t>21,521（9/14收）</t>
+        </is>
+      </c>
+      <c r="F126" s="55" t="inlineStr">
+        <is>
+          <t>報告日2026-09-15(Tue)，台股資料為2026-09-14(Mon)官方收盤；ADR、費半與全部美股個股為9/14美東收盤(台北9/15清晨)；期貨含今晨夜盤(TAIFEX標記9/15之盤後列，實際時段9/14 15:00至9/15 05:00)。
+(1)⚠️⚠️本報今日的內容同樣分成時序不同的兩段，且今天的分界比昨天更關鍵：第一段是9/14台股收盤(技術面與籌碼面雙雙確認轉弱)；第二段發生在台股收盤「之後」——美股半導體全面崩跌，且這一段尚未反映在任何台股價格中。本報立場自「中性偏空」下修為「看空」，並明確聲明這是技術面與籌碼面的下修，不是基本面的下修。
+(2)台股2330官方收NT$2,380(-30、-1.24%、開2,385／高2,395／低2,380、量21,521張、額NT$513.54億、189,734筆，TWSE STOCK_DAY確認)，連4日收黑。⚠️⚠️收盤價＝當日最低價，全日在前一日收盤之下運行、無下影線，代表盤中承接力量在收盤前未出現；與9/11「開盤即全日最高」同屬弱勢型態的兩種變形。高點連續第5個交易日降低(2,505→2,490→2,455→2,430→2,395)。⚠️同日加權指數僅-0.70%(收45,862.52)，台積電明顯弱於大盤、超額跌幅0.54個百分點——與9/11(台積電-1.63%vs大盤-1.61%、幾乎同幅)的情況相反。筆數189,734再創新高(較9/11的164,402增15.4%)，平均每筆僅0.11張(9/11為0.13張)，屬籌碼由法人向散戶移轉的特徵，通常不是落底訊號。
+(3)⚠️⚠️前一份日報所訂的三項檢核全部成立、且全部指向偏空：(a)外資賣超的持續性——9/14賣超11,191張(T86官方-11,191,022股)，不僅未收斂反而較9/11的8,251張再擴大35.6%，為9/2(-11,986,983股)以來最大單日賣超；連4日(9/9至9/14)合計賣超23,945張，已完全回吐9/7的16,135張與9/8的5,497張(合計21,632張)，本波外資買盤全數退場且倒賺2,313張。(b)前報列為「下一道未測試防線」的60MA季線2,399一日即失守，收盤低於季線19點且收在當日最低，為8/19(低於季線26.6點)以來最深；本報追蹤期間2330僅第11次收在季線之下。(c)前報預告「MACD紅柱若收斂速度不變將於下一個交易日前後翻黑」——9/14紅柱自+3.96轉為-4.77，準確兌現。
+(4)⚠️⚠️四項技術指標於同一日全部轉空，為本報追蹤期間首見：RSI(14)自50.02降至46.14(連4日下滑、正式跌破50多空分界)；MACD柱自+3.96翻黑至-4.77，且DIF 11.33下穿DEA 13.71構成標準死亡交叉；KDJ的J值自31.83暴跌33.97點至-2.14、跌破零軸，K(35.05)與D(53.64)負乖離自10.37點擴大至18.59點；股價2,380收在布林中軌2,410之下30點。⭐本報同時誠實標出兩項不該過度解讀之處：RSI 46.14距超賣區30仍有16點，屬「轉弱」非「超賣」；J值跌破0在本報追蹤期間多於1至3個交易日內引發技術性反彈——⚠️但反彈不等於止跌，7/17崩跌後即為反例。⭐均線：2,380已低於MA5 2,435、MA10 2,426、MA20 2,410、MA60 2,399四條，僅存MA120年線2,282(距現價-4.1%)。⚠️惟須指出一項機械性因素以免高估均線下彎的意義：MA5自2,451降至2,435(-16點)，其中約一半來自9/7的2,460滾出5日窗口；MA20僅自2,411微降至2,410(滾出8/17的2,400、滾入2,380)——目前是「價格離開均線」而非「均線帶著價格走低」。布林通道寬度5.35%(9/11為5.24%)幾乎持平，未見開口擴張。⭐技術指標口徑驗證：以同一套算法回算9/11已發布值(RSI 50.02／MACD柱3.96／K 52.57／D 62.94／J 31.83／MA5 2,451／MA20 2,411／布林2,474-2,411-2,348)全數完全複現，確認口徑未漂移。
+(5)⭐籌碼面除外資之外的兩項細節須分開看：投信轉買532張，為籌碼面唯一正面訊號，惟規模僅為外資賣超的4.8%，不足以對沖；自營商合計轉正+196張，但拆開看「自行買賣」仍為-33張、正值幾乎全部來自避險部位+229張——避險部位的增加通常對應選擇權與個股期的造市需求，不宜逕讀為自營商看多。三大法人分項加總合計賣超10,463張。外資近5日合計已轉為淨賣超18,448張。
+(6)⚠️⚠️⚠️第二段：台股收盤之後美股半導體全面崩跌，尚未反映在任何台股價格中。費半重挫-5.86%(-692.72點)收11,131.28，為本報追蹤期間單日最大跌幅。⭐跌幅分布極不平均，這本身就是判讀線索：設備四雄科林研發-8.29%、艾司摩爾-7.25%、應用材料-7.07%、科磊-6.39%，矽智財Arm-9.74%、封裝Amkor-8.91%；而台積電ADR僅-3.52%(收$418.01)、輝達-3.36%、高通-1.00%，蘋果甚至逆勢+0.24%(收$333.08，為本報19檔追蹤標的中唯一收紅)。台積電ADR相對費半的超額表現達+2.34個百分點。⭐判讀：本輪拋售重心在「AI資本支出的可持續性」(設備商營收直接對應客戶資本支出，故跌最重)，而非AI晶片的當期需求。美股四大指數：標普-0.48%收7,619.98、那斯達克-0.56%收26,186.41、道瓊-0.29%收52,421.20、VIX自15.84升至17.10(+7.95%)。
+(7)⭐成因是敘事而非數據，這決定了它的持續性難以預測：9/12(週末)Anthropic執行長Amodei發表文章呼籲AI業界「放緩腳步」，OpenAI的Altman與Musk相繼附和；一名離職Anthropic研究員稱AI公司拿人命當賭注的貼文獲逾1.5億次瀏覽，並有20多位美國國會議員呼籲加強監管(來源：NPR、CBS News、路透)。⚠️同期Michael Burry於9/12重申放空輝達等標的、類比1999至2000網路泡沫尾聲，美銀泡沫風險指標對半導體評分達0.91。⚠️第二層成因為利率：9/14美國10年期公債殖利率盤中一度觸及5.012%(2023年以來首見、終場收4.961%、9/11收4.975%)，布蘭特原油約每桶106美元。⚠️⚠️本報立場：這是情緒與評價事件，沒有任何一項涉及台積電的訂單、產能或定價；但正因為是敘事而非數據，它既可能一日反轉，也可能持續數週，本報不對其持續性作預測。
+(8)⭐⭐唯一的反向證據，也是本報沒有把立場推到「強烈看空」的主要理由：今晨夜盤已在完整看過美股9/14全場之後給出定價，結果並非跳空重挫。TAIFEX標記2026/09/15的盤後列(實際時段9/14 15:00至9/15 05:00)顯示，台積電個股期CDF 202609開2,370、最低2,368(一度低於現貨12點)後翻紅收2,387(+5、+0.21%)，⭐收盤反而高於現貨2,380達7點；台指期202609同時段收45,556(-221、-0.48%)，跌幅遠小於費半的-5.86%。⚠️惟夜盤量僅1,786口(約日盤12,523口的14%)，流動性低、指示性有限。
+(9)⭐期貨與選擇權：CDF 202609日盤收2,382(-34、-1.41%、開2,402／高2,402／低2,381、量12,523口、結算價2,382)，基差自+8點收斂至+2點正價差。未平倉自15,320口降至9,802口(-36.0%)，⚠️⚠️但這幾乎全是轉倉而非看空——9/16為9月月結算日，同期202610未平倉自12,820口增至18,576口(+44.9%)，兩者合計28,378口反而高於9/11的28,140口。TXO的P/C未平倉比0.88(賣權70,687口／買權80,290口、官方比率欄88.04%)。⚠️9/11為TXO週結算日，9/14為結算後重建首日，雙邊未平倉自112,666口回升至150,977口(+34.0%)屬機械性重建、不可跨日比較；⭐可讀的是重建後的結構比例——88.04%與9/11的87.70%幾乎一致，顯示急跌中並未出現恐慌性的賣權堆積，本欄屬中性。
+(10)⭐評價：TWSE官方BWIBBU 9/14顯示P/E 27.59x、P/B 9.59x、殖利率0.92%(9/11為27.94x／9.72x／0.91%)，財報基準維持115/2未變動。⭐算術自我檢核：P/E降幅-1.25%與股價跌幅-1.24%幾乎相同，確認分母未動、純為股價效果；以每股淨值248.05驗算2,380÷248.05＝9.595≈9.59，與官方值相符。市值約NT$61.7兆。ADR端P/E約30.7x、P/B約10.7x(依比例換算、非官方申報)。⚠️⚠️本日須補充一項與評價直接相關的外部發展：9/14拋售的敘事核心正是「AI相關類股評價過高」——本欄各項百分位數(P/E位於5年約88百分位、10年約89百分位、P/B約92百分位)本身即顯示評價處於歷史高檔，此前被高獲利成長合理化；一旦市場對AI資本支出的持續性產生懷疑，高百分位就會由「成長溢價」轉為「回檔風險」。⚠️百分位欄位為既有估算、非每日重算。
+(11)⭐ADR溢價自13.72%收斂至11.28%(-2.44個百分點)，方向與前一日完全相反、但成因同樣是時間差而非評價：理論平價＝5×2,380÷31.68＝375.63(採捨入後匯率)，對市價418.01之溢價+11.28%。⭐9/11溢價之所以擴大到13.72%，是因為ADR已先反映了台股收盤後才公布的美國8月CPI利多；9/14美股一轉為半導體重挫，ADR單日-3.52%而台股僅-1.24%，溢價便隨之收斂——即ADR正在向下補回它先前多漲的部分。⚠️⚠️惟收斂後的+11.28%仍遠高於本報追蹤期間常見的5至8%區間，意味這一輪的時間差尚未完全消化完畢。⭐相對強弱：近5日-3.25%(基準9/7收2,460)，大盤近5日-3.09%；近1月-0.63%(基準日曆同日8/14收2,395，⚠️基準每日移動、本欄的轉負有一部分來自基準日更換)，大盤+0.11%；YTD+50.2%(基準2026-01-02收1,585)，落後大盤+56.3%與費半+51.1%。
+(12)⚠️匯率連3日走貶：新台幣9/14交易日收31.676(本報採31.68)，較9/11的31.635再貶0.13%，⭐方向對台積電以美元計價的營收換算有利，惟幅度小、對本日股價不構成解釋力。⚠️取數限制：本欄採Yahoo TWD=X的當日K棒收盤而非銀行間16:00定盤價，兩者通常差距在0.01以內(9/11本報採31.63、日K棒為31.635，可相互印證)，但並非同一口徑。今晨9/15 09:18台北盤中報31.729，續貶方向未變，屬盤中值不納入計算。
+(13)⭐台股供應鏈9/14(尚未反映美股當日重挫)：華邦電-6.71%收160.00元(連4日下跌、為台股追蹤標的中跌幅最大)、聯發科-0.55%收4,560元、日月光-0.97%收612.00元(相對抗跌，惟其美股同業Amkor同日崩跌-8.91%、時序不同)。韓股9/14：三星電子-4.05%收249,000韓元、SK海力士-6.35%收1,697,000韓元(⚠️採9/14收盤，非今晨盤中價)。
+(14)⭐台積電自身無新事件：本報於9/12至9/15窗口內未查獲台積電的新財報、產能、訂單或定價公告，唯一相關項目為Susquehanna於9/12重申「買進」評等(例行更新、未附新目標價)；客戶端(輝達、蘋果、超微、博通、高通)同期亦無獨立新業務公告，股價波動全部來自類股連動。⚠️本報明確指出此點的用意在於：9/14台積電ADR的-3.52%與台股9/14的-1.24%，沒有任何一部分來自公司基本面的變化。最近一項基本面數據仍是9/10公布的8月營收NT$5,148.1億(+53.3% YoY、+10.1% MoM，單月首度突破5,000億元大關)，下一個基本面檢核點為10月中旬的Q3法說會。
+(15)⚠️⚠️本週三9/16(僅剩1個交易日)雙事件同日發生，性質互不相關但極易互相污染判讀：(a)台股2330除息，每股現金股利NT$7.00001(TWSE官方除權除息預告表TWT48U，本日以查詢區間2026-09-01至10-31第四度查得，2330為該區間68筆之一，申報基準115年第2季、每股淨值248.05、每股盈餘49.33，四日數字完全一致)；以9/14收盤2,380計除息參考價約2,373，股價機械性扣除約7點(-0.29%)，P/E與P/B同步機械性下降——讀者比較9/16之後的股價時務必還原此缺口。(b)9/16為2026年9月第三個週三，即台指期貨與選擇權月結算日；選擇權未平倉將大幅結清重建，台指期與個股期換月至202610合約，未平倉躍升屬轉倉而非新增部位，新舊合約價格不可跨合約比較。⭐ADR股利金額維持既有結論：NT$7.00001×5÷匯率約31.42≈US$1.114，與CNBC所載一致；⚠️台積電IR官網(investor.tsmc.com)持續回HTTP 403、未能取得一手公告，故標示為【以台股股利換算，待官方確認】。12/10為8/11董事會核准之Q2 2026股利(NT$7.0/股、基準日12/16)除息日，屬不同批次。
+(16)⚠️⚠️FOMC於9/15至16開會，利率決策於台北時間9/17凌晨2:00公布。⚠️本項本日出現重大變化、須明確更正讀者可能的既有預期：市場目前主流預期是「升息」而非降息，惟各來源機率差異極大——摩根大通財富管理與高盛的基準情境為升息1碼、期貨隱含機率約80至87%，但CME FedWatch約56%、Kalshi約48%、Polymarket約49%；前克里夫蘭聯準銀行總裁Mester表示「市場隱含機率看起來比我自己會給的高」。⭐本報未能證實何者較準確，故以「看法分歧、介於5成至8成多」並陳，不取單一數字。⚠️若升息成真並疊加AI資本支出疑慮，對本益比位於5年約88百分位的台積電將形成評價與資金的雙重壓力；反之若按兵不動，則可能成為本輪情緒反轉的觸發點。
+(17)⭐⭐今日檢核價位訂為兩個，明日將逐條回頭驗證：(a)下檔看2,375(8/24收盤＝本波前低)，若收在其下，則「跌破季線」升級為「波段轉折」；(b)上檔看2,399(60MA季線)，若能收復，則9/14的跌破可改判為單日假跌破。第一順位觀察為台股對美股9/14崩跌的補跌幅度——若跌幅明顯小於ADR的-3.52%，可確認本輪拋售對晶圓代工的衝擊有限；第二順位為外資賣超規模，若再現萬張以上賣超，籌碼面即由「回檔」轉為「趨勢性撤出」。⚠️須誠實聲明：本報「看空」是對未來1至5個交易日技術面與籌碼面的判斷，不含對台積電基本面的負面看法——8月營收創新高、連11季超預期、Q3法說會預計10月中旬，這些基本面事實在本輪下跌中沒有任何一項改變。</t>
+        </is>
+      </c>
+      <c r="G126" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:G2"/>

</xml_diff>

<commit_message>
@ daily: 2026-09-16 日報 HTML & Excel 更新
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
@
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -189,7 +189,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -249,6 +249,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E9F2FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -329,7 +334,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -505,6 +510,18 @@
     </xf>
     <xf numFmtId="0" fontId="28" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -895,7 +912,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-09-15</t>
+          <t>報告更新日期：2026-09-16</t>
         </is>
       </c>
     </row>
@@ -2571,7 +2588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="36" min="1" max="1"/>
@@ -2825,135 +2842,162 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="22" t="inlineStr">
+      <c r="A15" s="62" t="inlineStr">
+        <is>
+          <t>2026 年 9 月批次</t>
+        </is>
+      </c>
+      <c r="B15" s="63" t="inlineStr">
+        <is>
+          <t>NT$7.00001</t>
+        </is>
+      </c>
+      <c r="C15" s="64" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="D15" s="64" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="E15" s="65" t="inlineStr">
+        <is>
+          <t>Source: TWSE 官方除權除息預告表 TWT48U（2026-09-16 取得，申報基準 115 年第 2 季、每股淨值 248.05、每股盈餘 49.33）；配息基準日 2026-09-22。除息參考價算術值 2,377.99999，依 TWSE 升降單位取整後開盤競價基準 2,380。ADR 端同日（美東）除息 US$1.114。⚠️ 季度歸屬未由 TSMC IR 一手公告確認（investor.tsmc.com 持續回 HTTP 403），故本列以除息批次標示、不逕行標註季別。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="22" t="inlineStr">
         <is>
           <t>Q1 2026</t>
         </is>
       </c>
-      <c r="B15" s="23" t="inlineStr">
+      <c r="B16" s="23" t="inlineStr">
         <is>
           <t>NT$6.00</t>
         </is>
       </c>
-      <c r="C15" s="25" t="inlineStr">
+      <c r="C16" s="25" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
       </c>
-      <c r="D15" s="25" t="inlineStr">
+      <c r="D16" s="25" t="inlineStr">
         <is>
           <t>2026-04</t>
         </is>
       </c>
-      <c r="E15" s="26" t="inlineStr">
+      <c r="E16" s="26" t="inlineStr">
         <is>
           <t>Source: TSMC IR</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="20" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="20" t="inlineStr">
         <is>
           <t>Q4 2025</t>
         </is>
       </c>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>NT$4.50</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>2026-01</t>
         </is>
       </c>
-      <c r="E16" s="8" t="inlineStr">
+      <c r="E17" s="8" t="inlineStr">
         <is>
           <t>Source: TSMC IR</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="21" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="21" t="inlineStr">
         <is>
           <t>Q3 2025</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>NT$4.50</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>2025-10</t>
         </is>
       </c>
-      <c r="E17" s="11" t="inlineStr">
+      <c r="E18" s="11" t="inlineStr">
         <is>
           <t>Source: TSMC IR</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="20" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="20" t="inlineStr">
         <is>
           <t>Q2 2025</t>
         </is>
       </c>
-      <c r="B18" s="6" t="inlineStr">
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>NT$4.50</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>2025-07</t>
         </is>
       </c>
-      <c r="E18" s="8" t="inlineStr">
+      <c r="E19" s="8" t="inlineStr">
         <is>
           <t>Source: TSMC IR</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="21" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="21" t="inlineStr">
         <is>
           <t>Q1 2025</t>
         </is>
       </c>
-      <c r="B19" s="9" t="inlineStr">
+      <c r="B20" s="9" t="inlineStr">
         <is>
           <t>NT$4.50</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="D20" s="3" t="inlineStr">
         <is>
           <t>2025-04</t>
         </is>
       </c>
-      <c r="E19" s="11" t="inlineStr">
+      <c r="E20" s="11" t="inlineStr">
         <is>
           <t>Source: TSMC IR</t>
         </is>
@@ -3333,7 +3377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G126"/>
+  <dimension ref="A1:G127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3355,7 +3399,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-09-15</t>
+          <t>最後更新：2026-09-16</t>
         </is>
       </c>
     </row>
@@ -8006,6 +8050,60 @@
         </is>
       </c>
     </row>
+    <row r="127">
+      <c r="A127" s="50" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B127" s="50" t="inlineStr">
+        <is>
+          <t>NT$2,385（9/15收）</t>
+        </is>
+      </c>
+      <c r="C127" s="51" t="inlineStr">
+        <is>
+          <t>+0.21%（9/15收）</t>
+        </is>
+      </c>
+      <c r="D127" s="50" t="inlineStr">
+        <is>
+          <t>US$413.75（9/15收）</t>
+        </is>
+      </c>
+      <c r="E127" s="50" t="inlineStr">
+        <is>
+          <t>15,216（9/15收）</t>
+        </is>
+      </c>
+      <c r="F127" s="52" t="inlineStr">
+        <is>
+          <t>報告日2026-09-16(Wed)，台股資料為2026-09-15(Tue)官方收盤；ADR、費半與全部美股個股為9/15美東收盤(台北9/16清晨)；期貨含今晨夜盤(TAIFEX標記9/16之盤後列，實際時段9/15 15:00至9/16 05:00)。
+(0)⚠️⚠️三項閱讀前提請先看過，否則本行數字必被誤讀：(a)本行所載台股收盤2,385為除息前(含息)最後一個收盤價——台股2330於今日9/16除息每股NT$7.00001，今日起的股價與2,385不可直接相減，須先還原除息缺口；(b)9/15的量能萎縮有明確的機械性成因(漢測申購凍資，詳(6))，不可讀為買盤退場；(c)今日9/16同為9月台指期貨與選擇權月結算日，明日的未平倉、量能與法人籌碼數據皆不可與今日直接比較。
+(1)⭐台股2330官方收NT$2,385(+5、+0.21%、開2,405＝全日最高／低2,380＝9/14收盤／量15,216張、額NT$363.76億、84,331筆，TWSE STOCK_DAY確認)，連4日收黑中止。⭐K線型態須兩面並陳：正面是全日最低2,380恰為前一日收盤、全程未跌破，且收盤高於最低5點留有下影線，與9/14的無下影線收最低相反；保留是開盤2,405即為全日最高，高開後追價力量同樣不足、全日僅收復5點，屬「止跌」而非「反攻」。⭐本日中止了一項連5個交易日的偏空證據：高點序列2,505→2,490→2,455→2,430→2,395連5日降低，9/15的2,405為9/8以來首次高點不再降低。⭐同日加權指數收45,511.49(-351.03、-0.77%)，台積電逆勢收紅、超額+0.98個百分點，與9/14(落後0.54個百分點)方向完全相反。本報立場自「看空」回調為「中性偏空」。
+(2)⭐逐條履行前一份日報所訂四項檢核，結果為二項偏多、一項偏空、一項未觸發：(a)前報第一順位「台股跌幅是否小於ADR的-3.52%」——不只小於而是完全未補跌，收+0.21%，以最強形式通過；(b)前報第二順位「2,375(8/24收盤＝本波前低)的得失」——全日最低2,380，未觸及即守住；⚠️惟另一半條件「收復60MA季線2,399」未達成(收2,385、仍低12點)，故9/14的季線跌破尚不能改判為單日假跌破，維持「已跌破、待收復」；(c)前報第三順位「若再現萬張以上外資賣超即升級為趨勢性撤出」——外資賣超4,226張，遠低於門檻，升級條件未觸發；(d)前報所引今晨夜盤個股期收2,387，與現貨實收2,385僅差2點，夜盤指示性獲驗證。
+(3)⭐⭐籌碼面是本日唯一通過對照組檢驗的實質正面訊號：外資9/15賣超4,226張(TWSE T86官方買進7,484,872股／賣出11,711,632股／淨-4,226,760股，依既定口徑向零截斷)，較9/14的11,191張收斂62.2%，為本波連5日賣超中最小的一日。⭐關鍵在於本報沒有停在這個數字：量縮日的籌碼收斂必須先排除「全市場流動性萎縮」這個機械性成因，故另抓TWSE BFI82U全市場三大法人買賣金額作對照組——結果是9/15全市場外資賣超NT$627.0億，反而較9/14的NT$369.6億擴大69.6%。⭐⭐結論明確且可複算：在外資加碼賣出台股整體的同一天，台積電的賣超規模腰斬，屬賣壓自台積電輪出，而非流動性造成的假收斂。⚠️保留：連5日(9/9至9/15)外資合計仍賣超28,171張。投信小幅轉賣13張(-13,848股)；自營商合計+350張(自行買賣+267,050股→+267張、避險+83,497股→+83張，267+83=350與官方合計換算一致)，與9/14相反、正值主要來自自行買賣。三大法人分項加總合計賣超3,889張(官方合計欄-3,890,061股換算-3,890，差1張屬正常捨入)。
+(4)⚠️⚠️技術面與價格背道而馳，這是本報不轉為中性的主因：價格漲5點，四項指標卻有兩項續惡化、兩項僅止穩。(a)⚠️⚠️MACD柱自-4.77擴大至-9.61(兩個交易日內翻倍)，DIF自11.33急降至7.71、DEA自13.71降至12.51，DIF下滑速度為DEA的3倍，負乖離自-2.38擴大至-4.80——9/14成立的死亡交叉不僅未修復反而加深，為本日最強的偏空證據。(b)⚠️⚠️KDJ的J值自-2.14再降至-13.89(連2日低於零軸)，K自35.05降至24.70、D自53.64降至44.00，K-D負乖離自-18.59擴大至-19.30。⭐成因可複算：9日窗口為9/3至9/15，窗口內最高價仍為9/8的2,505、最低價2,380(9/3、9/14、9/15三日同值)，故RSV=(2,385-2,380)÷(2,505-2,380)×100=4.0，K=35.05×2/3+4.0/3=24.70、D=53.64×2/3+24.70/3=44.00、J=3K-2D=-13.89；⚠️只要2,505仍留在9日窗口內(依交易日推算將續留至9/18)，分母就維持125點高檔、RSV難以回升，KDJ因此有相當程度是滾動窗口造成的機械性受壓。(c)⭐RSI(14)自46.14微升至46.88，中止連4日下滑，惟仍在50之下、距超賣區30尚有近17點，屬「止穩」非「轉強」。(d)⭐股價2,385仍低於布林中軌2,410達25點(前一日低30點)，通道寬度5.31%(9/14為5.35%)連2日微收、未見開口擴張。
+(5)⭐均線變化須先剝除機械性成因，否則會高估惡化程度：(a)⭐⭐MA5自2,435大幅下滑至2,418(-17點)，但這17點100%來自滾動窗口效應——滾出9/8的2,470、滾入2,385，(2,385-2,470)÷5恰為-17.0，與本日上漲5點完全無關；(b)⭐MA20自2,410.0微升至2,410.25(滾出8/18的2,380、滾入2,385)，中期均線仍在極緩上行、並未下彎，「價格離開均線」而非「均線帶著價格走低」的判斷較前一日更明確；(c)⚠️MA60季線自2,399降至2,397，收2,385仍低於季線12點、跌破狀態未解除，惟距離自19點收斂至12點，且收斂的一半來自季線自身下移；(d)⭐MA120年線自2,282升至2,287(距現價-4.1%)，為唯一仍在價格下方的均線。⭐技術指標口徑驗證：以同一套算法回算9/14已發布值(RSI 46.14／MACD柱-4.77／DIF 11.33／DEA 13.71／K 35.05／D 53.64／J -2.14／MA5 2,435／MA10 2,426／MA20 2,410／MA60 2,399／MA120 2,282／布林2,474-2,410-2,346／5日均量21,844)全數逐項完全複現，確認口徑未漂移。序列為TWSE官方2026-01-02至2026-09-15共170個交易日。
+(6)⚠️⚠️本日最須警惕的認知陷阱，同時影響量能與價格兩個判讀：9/15成交量15,216張(較9/14的21,521張減29.3%)、全市場成交值NT$6,347.07億，經本報比對TWSE FMTQIK官方序列為2026年170個交易日中第3低(僅高於4/07的5,846.92億與1/12的6,264.08億)。⭐成因是機械性的資金凍結——興櫃股王漢測(7856)9/10至9/14公開申購，凍結市場資金達NT$8,656.13億元、38萬4,717筆申購、中籤率0.27%，創台股凍資紀錄(前次紀錄為鴻勁精密的近3,000億元)；漢測9/22掛牌上櫃、承銷價每股2,250元，9/16上午電腦抽籤、9/17解交股款。⚠️故量能門檻本日字面未過(15,216張較5日均量19,101張低20.3%)但成因已確認為機械性，不列為偏空證據；⚠️同時必須誠實指出反面——在極低流動性下形成的+0.21%上漲，其訊號強度也應同步折價，真正的檢驗要等9/17資金解凍之後。⭐另註：媒體報導之成交值6,034.53億元與「今年次低」係採較窄口徑，本報一律採TWSE FMTQIK官方值6,347.07億元並自行比對全年序列。
+(7)⚠️⚠️美股端9/15出現方向分歧，且台積電ADR站在較弱的一邊，這是本報不轉為中性的第二個理由：費半止跌反彈+0.40%(+44.27點)收11,175.55(盤中高11,304.24、低11,128.88)。⚠️⚠️重點不在漲幅而在結構——反彈完全由9/14跌最重者主導(高通+4.25%、超微+2.19%、Arm+1.18%、艾司摩爾+1.04%、輝達+0.57%、美光+0.39%)，屬典型超跌修復而非趨勢重啟；兩日合計費半仍-5.48%、僅收復9/14跌幅的約7%。⚠️而台積電ADR收$413.75(-1.02%)、博通-1.58%、Amkor-1.57%、蘋果-0.52%續跌；台積電ADR相對費半超額-1.42個百分點，與9/14領先2.34個百分點完全反轉。⭐兩日合計台積電ADR -4.50%，在19檔追蹤標的中屬中段(Amkor -10.34%、科林研發-9.17%、Arm -8.67%最深；蘋果-0.28%、超微-2.31%、輝達-2.80%最淺)——即台積電既未被當成本輪拋售的核心，也未被當成避風港。⚠️同期大盤反而續跌：標普-0.45%收7,585.73、那斯達克-0.78%收25,981.57、VIX 17.20(+0.58%)；10年期公債殖利率收4.996%、盤中觸及5.016%再創新高；布蘭特原油升至每桶約108美元(媒體歸因美伊緊張再起)。⚠️本日多檔美股個股的日K棒close欄為null，本報依既定作法改採Yahoo meta.regularMarketPrice並逐檔驗證時間戳(均為2026-09-15 20:00 UTC＝美東16:00收盤)，非採用盤中價。
+(8)⭐期貨與選擇權(⚠️今日9/16為9月月結算日，以下數字明日起皆不可跨日比較)：個股期CDF 202609日盤收2,392(+10、+0.42%、開2,384／高2,407／低2,383、量11,452口、結算價2,392)，漲幅大於現貨的+0.21%；基差自+2點擴大至+7點正價差，為連3日收斂後首次擴大，⚠️惟結算前基差本就會向結算價收斂、指示性低於平日。未平倉7,291口，自9/14的9,802口再減25.6%，⚠️⚠️幾乎全屬轉倉——同期202610自18,576口增至22,796口(+22.7%)，兩者合計30,087口反較9/14的28,378口增加6.0%。TXO未平倉P/C比0.86(賣權81,556口／買權94,956口、官方比率欄85.89%)，較9/14的88.04%降2.15個百分點、為9/10(82.67%)以來最低，連4日落在80至90%區間；⭐買權未平倉增幅18.3%大於賣權的15.4%，即結算前部位建立略偏買權一側，與外資賣超收斂、正價差回升同向，屬中性偏多但量級小。⭐今晨夜盤未給出方向：TAIFEX標記2026/09/16的盤後列(實際時段9/15 15:00至9/16 05:00)顯示CDF 202609開2,385、高2,391、低2,379、收2,386(+1、+0.04%、量1,356口)，與現貨2,385幾乎平價、未見方向性跳空；台指期202609收45,529(-63、-0.14%、量22,905口)。⚠️夜盤量僅為日盤的11.8%，且今日為結算日、部位多屬結算前調整，指示性有限。
+(9)⭐評價：TWSE官方BWIBBU 9/15顯示P/E 27.65x、P/B 9.61x、殖利率0.92%(9/14為27.59x／9.59x／0.92%)，財報基準維持115/2未變動。⭐算術自我檢核：P/E升幅+0.22%與股價漲幅+0.21%幾乎相同，確認分母未動、純為股價效果；以每股淨值248.05驗算2,385÷248.05＝9.6151≈9.61，與官方值相符。市值約NT$61.8兆。ADR端P/E約30.4x、P/B約10.6x(依官方值×ADR溢價係數1.1006換算、非官方申報值)。⚠️⚠️預告一項明日必然發生的機械性變動：今日除息NT$7.00001後，P/E與P/B將同步機械性下降約0.29%(P/E約至27.57x、P/B約至9.58x)，與評價重估無關。⚠️外部評價風險維持前一版提醒：9/14拋售的敘事核心正是「AI相關類股評價過高」，本報P/E位於5年約88百分位、10年約89百分位、P/B約92百分位，屬歷史高檔(百分位為既有估算、非每日重算)。
+(10)⭐ADR溢價自11.28%續收斂至10.06%(-1.22個百分點)，為連續第2日收斂，成因單純且可複算：理論平價＝5×2,385÷31.72＝375.95(採捨入後匯率)，對市價413.75之溢價+10.06%；台股+0.21%(分母升)、ADR-1.02%(分子降)，兩者反向而行必然壓縮溢價，屬時間差的持續消化而非評價重估。⚠️⚠️惟收斂後的+10.06%仍明顯高於本報追蹤期間常見的5至8%區間，時間差尚未消化完畢。⭐⭐預先提醒明日起的計算陷阱：台股2330於9/16(台北)除息NT$7.00001、ADR亦於9/16(美東)除息US$1.114，兩端除息日雖同標9/16卻分屬不同時區的交易日，明日計算溢價時兩邊缺口必須同時還原，否則會出現虛假跳動。⭐相對強弱：近5日-3.44%(基準9/8收2,470)，大盤近5日-3.38%；近1月-0.42%(基準日曆同日9/15對8/15，因8/15為週六故取前一交易日8/14收2,395，與前一份日報基準日相同，故本日1個月報酬由-0.63%收斂至-0.42%全部來自本日上漲、不含基準移動效果)，大盤-0.65%；YTD+50.5%(基準2026-01-02收1,585)，落後大盤+55.1%與費半+51.7%。
+(11)⚠️匯率連4日走貶：新台幣9/15交易日收31.7176(本報採31.72)，較9/14的31.676再貶0.13%，四日累計自31.464貶值0.81%。⭐累計幅度已自「雜訊」升級為「可觀察」：0.81%對毛利率影響約+32bps，方向對台積電以美元計價的營收換算有利。⚠️取數限制：本欄採Yahoo TWD=X的當日K棒收盤而非銀行間16:00定盤價，兩者通常差距在0.01以內但並非同一口徑。⭐今晨9/16台北09:15前後盤中報31.851，較9/15收盤再貶0.42%、單日幅度為四日來最大，屬盤中值不納入計算，明日回頭確認。
+(12)⭐台股供應鏈9/15(部分標的對美股9/14崩跌作出遞延補跌)：日月光-3.27%收592.00元(跌破600元關卡、為台股追蹤標的中跌幅最大，成因為其美股同業Amkor已於9/14崩跌-8.91%、日月光當日僅跌0.97%尚未反映)；聯發科-2.85%收4,430元(連3日下跌、跌幅較9/14的-0.55%顯著擴大)；華邦電-0.31%收159.50元(連5日下跌但跌幅自9/14的-6.71%大幅收斂)。⚠️值得注意的是日月光與聯發科確實補跌，而台積電完全未補跌，兩者形成鮮明對照。韓股9/15收盤：三星電子-0.20%收248,500韓元、SK海力士-0.41%收1,690,000韓元(兩者跌幅均自9/14的-4.05%與-6.35%大幅收斂)；⭐今晨9/16台北09:00前後韓股盤中回升——SK海力士1,721,000韓元(+1.83%)、三星250,750韓元(+0.91%)，為本日所見最強的亞洲盤領先訊號之一，惟屬盤中值僅供參考。
+(13)⭐台積電自身無新業務事件：本報於9/15至9/16窗口內未查獲台積電的新財報、產能、訂單或定價公告，官網新聞稿亦無新增項目。周邊可記錄者有二：(a)媒體報導台積電與三星均已承諾採用艾司摩爾最新世代機台、AI需求驅動設備支出——⚠️本報誠實界定：該報導與台積電9/2 SEMICON所揭露的2026資本支出上修至600至640億美元、設備需求達2025年底預估1.9倍的方向一致，但未提供新的量化承諾，不改變既有判讀；(b)博通於VMware Explore 2026發表多項企業級AI產品，惟股價當日仍收-1.58%，媒體歸因為公債殖利率與油價走升的整體避險情緒而非公司事件。最近一項基本面數據仍是9/10公布的8月營收NT$5,148.1億(+53.3% YoY、+10.1% MoM)，下一個基本面檢核點為10月中旬的Q3法說會與10/10前後的9月營收。
+(14)⭐⭐今日9/16除息詳情：台股2330除息每股現金股利NT$7.00001(TWSE官方除權除息預告表TWT48U，本日以查詢區間2026-09-01至12-31再次查得，2330為該區間62筆之一，申報基準115年第2季、每股淨值248.05、每股盈餘49.33，與前四日查得完全一致)。⭐除息參考價：算術值為2,385-7.00001=2,377.99999，依TWSE升降單位規定(股價1,000元以上為5元)四捨五入後開盤競價基準為2,380——以2026-04-09前例驗證此取整慣例：前收1,950-1.50=1,948.50→基準1,950，當日收1,955標為+5.00。⚠️除息比率0.29%；證交所估算本次除息使加權指數基準下調約55.64點(約-0.12%)。⭐本次為台積電首度季配息達7元；配息基準日9/22、現金股利預計10/8發放。⭐填息歷史供參：自2019 Q3改採季配息以來共除息28次，其中22次(79%)於除息當日即完成填息，最近4次全數當日填息。⭐ADR端同步於9/16(美東時間)除息每ADR US$1.114(NT$7.00001×5÷匯率約31.42≈US$1.114，與CNBC所載一致)。⭐下一批為12/10除息NT$7.0/股、2027-01-07發放(來源為8/11董事會決議與媒體報導)；⚠️該筆尚未出現在TWT48U預告表9/1至12/31區間的回傳結果中，屬預告表尚未登錄之未來事件。
+(15)⚠️⚠️FOMC於9/15至16開會，利率決策於美東9/16 14:00、即台北時間9/17凌晨2:00公布，Fed主席Warsh於14:30記者會。⚠️本項自前一份日報以來出現重大變化、須明確更正讀者的既有預期：升息1碼的機率估計已自本報上一版所載的48%至87%分歧區間，大幅上修並收斂至約90%(defirate預測市場90.3%、維持不變8.7%；centralbank.watch所示市場隱含約91%)。驅動因素為通膨未如預期降溫、以及美伊衝突推升的能源成本，7月會議已有三位委員投下贊成升息的反對票。⚠️惟機構看法仍分歧：摩根大通財富管理已改為預期升息1碼，高盛則稱9月升息「非常不可能」並預期全年按兵不動。⭐本報未能證實何者較準確，如實並陳、不取單一數字。⚠️若升息成真並疊加AI資本支出疑慮，對本益比位於5年約88百分位的台積電將形成評價與資金的雙重壓力；反之若按兵不動或釋出鴿派訊號，則可能成為本輪情緒反轉的觸發點。
+(16)⭐⭐今日檢核價位訂為兩個，明日將逐條回頭驗證，⚠️且兩者都已還原除息缺口、請勿與9/15收盤2,385直接比較：(a)填息檢核——今日開盤競價基準2,380，若收盤回到2,385之上即完成當日填息，符合近4次除息全數當日填息的歷史型態；⚠️反之若未能填息，則9/15的止跌訊號應被追認為流動性造成的假象；(b)季線檢核——除息後的60MA季線約落在2,395附近，收復與否仍是本波能否改判的關鍵。⭐其他優先觀察項：動能與價格的背離是否收斂(若MACD負柱續擴大至-13以上，則9/15的上漲應被追認為反彈失敗)；外資賣壓輪出的持續性(若今日台積電賣超重返萬張，則9/15的收斂須改判為凍資期的流動性假象)。⚠️須誠實聲明：本報「中性偏空」是對未來1至5個交易日技術面與籌碼面的判斷，不含對台積電基本面的負面看法——8月營收創新高、連11季超預期、Q3法說會預計10月中旬，這些基本面事實在本輪修正中沒有任何一項改變。</t>
+        </is>
+      </c>
+      <c r="G127" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:G2"/>

</xml_diff>

<commit_message>
daily: 2026-09-17 日報 HTML & Excel 更新
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -912,7 +912,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-09-16</t>
+          <t>報告更新日期：2026-09-17</t>
         </is>
       </c>
     </row>
@@ -3377,7 +3377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G127"/>
+  <dimension ref="A1:G128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3399,7 +3399,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-09-16</t>
+          <t>最後更新：2026-09-17</t>
         </is>
       </c>
     </row>
@@ -8104,6 +8104,58 @@
         </is>
       </c>
     </row>
+    <row r="128">
+      <c r="A128" s="53" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B128" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,380（9/16收，除息後）</t>
+        </is>
+      </c>
+      <c r="C128" s="54" t="inlineStr">
+        <is>
+          <t>+0.08%（9/16收，對除息參考價2,377.99）</t>
+        </is>
+      </c>
+      <c r="D128" s="53" t="inlineStr">
+        <is>
+          <t>US$417.72（9/16收）</t>
+        </is>
+      </c>
+      <c r="E128" s="53" t="inlineStr">
+        <is>
+          <t>20,919（9/16收）</t>
+        </is>
+      </c>
+      <c r="F128" s="55" t="inlineStr">
+        <is>
+          <t>報告日2026-09-17(Thu)，台股資料為2026-09-16(Wed)官方收盤；ADR、費半與全部美股個股為9/16美東收盤(台北9/17清晨)；期貨含今晨夜盤(TAIFEX標記9/17之盤後列，實際時段9/16 15:00至9/17 05:00，涵蓋FOMC宣布時點)。
+(0)⚠️⚠️三項閱讀前提請先看過，否則本行所有數字必被誤讀：(a)9/16為除息日，台積電每股配發NT$7.00001，TWSE官方TWT49U三基準值為除權息前收盤價2,385.00、除息參考價2,377.99、開盤競價基準2,380.00；本行台股所有價格與報酬率若未註明「還原除息」一律為未還原原始價，與9/15以前不可直接相減。(b)9/16同為2026年9月台指期貨與選擇權月結算日，選擇權未平倉大規模結清重建、個股期主力合約自202609換月至202610，未平倉與價格皆為新基期，變動幅度不可與前一日比較。(c)美國聯準會於台北時間9/17凌晨宣布升息1碼，本行美股與ADR數據均已包含該事件反應。
+(1)⭐⭐本日最重要的事是聯準會升息：FOMC於美東9/16宣布調升聯邦資金利率目標區間1碼、自3.50-3.75%上調至3.75-4.00%，12票對0票一致通過(來源為Fed官網9/16聲明稿原文，本報直接調閱原始新聞稿確認、非引用二手報導)。聲明指出經濟活動穩健擴張、生產力強勁，但通膨仍偏高，升息是為使通膨更及時回到2%目標。⭐市場首日反應與直覺相反：費半收11,246.11(+0.63%)、台積電ADR收$417.72(+0.96%)、Intel+4.03%、AMD+1.65%，升息未壓抑半導體風險偏好。⚠️但標普500收7,551.81(-0.45%)、那斯達克25,978.42(-0.01%)、VIX升至17.71(+2.97%)，大盤與半導體明顯分歧，首日反應不足以定調。⚠️後續升息路徑的點陣圖細節本報未能自官方聲明稿取得，列為未能證實。
+(2)⭐台股2330官方收NT$2,380(開2,375＝全日最低／高2,395／量20,919張、額NT$498.13億、142,588筆，TWSE STOCK_DAY確認)。⚠️TWSE的漲跌價差欄於除權息日標示為X0.00，X為「除權息、不計算漲跌」之註記而非數值0——本報已用2026-03-17前例驗證(當日同標X0.00但收1,870對前一日1,845實為上漲)。⭐對除息參考價2,377.99而言本日為+2.01(+0.08%)。⭐⭐填息判定：收2,380高於參考價2.01元、填息2.01÷7.00001＝28.7%，⚠️但未回到除息前收盤2,385，本報認定當日未完成填息，中止近4次除息全數當日填息的型態。⭐惟須公允並陳兩點：收盤仍在參考價之上、未出現貼息；且盤中最高2,395已超越2,385達10元，盤中一度完成百分之百填息。⚠️全日振幅20元(2,375-2,395、0.84%)屬偏低的一端，但並非9月最小——9/14的15元更小，9/03與9/10同為20元；本報判讀為觀望而非多空激戰。⭐盤中最低2,375恰為8/24收盤＝本波前低，本報自9/11起列為關鍵下檔的該價位本日首度受實際測試並守住。
+(3)⭐逐條履行前一份日報所訂四項檢核，結果為一項未通過、一項字面成立但實質未成立、一項字面未達但實質延續、一項如期發生：(a)第一順位「當日完成填息」——未通過，理由見(2)。(b)第二順位「MACD負柱是否擴大至-13以上」——本日-13.00恰觸門檻，⭐⭐但以還原除息的對照組(9/16收盤視為2,387)重算為-12.11、未達門檻，本報判定「字面成立、實質未成立」，不逕行追認9/15上漲為反彈失敗，門檻順延至9/17在無除息干擾的乾淨基礎上重判。(c)第三順位「外資賣超是否重返萬張」——8,744張、字面未達，⭐⭐但實質上比萬張更重要，理由見(4)。(d)第四順位「月結算與換月」——如期發生，數據見(7)。
+(4)⭐⭐⭐籌碼面本日有一項必須用對照組才能看懂、且方向與字面相反的事實：外資對台積電單日賣超8,744張(TWSE T86官方買進8,374,396股／賣出17,118,776股／淨-8,744,380股，依既定口徑向零截斷)，以2,380元計約NT$208.1億；⚠️⚠️而同日TWSE BFI82U顯示全市場外資淨賣超僅NT$179.8億——即台積電一檔的賣超金額「超過」全市場外資淨賣超總額，換算下來外資對台積電以外的台股合計為淨買超約NT$28億。⭐與9/15的型態方向一致但強度加倍：9/15台積電賣超100.8億、全市場627.0億，占16%；9/16占比升至116%。⭐本報據此認定「資金自台積電輪出至其他台股」已連續2個交易日成立，符合前報所訂「背離延續兩日以上可確認為資金輪出」的條件。⚠️惟必須誠實並陳第二成因：9/16為除息日，外資基於台灣股利所得扣繳(本日已由ADR端股利調整反推實際扣繳率約21%)本就傾向在除息日前後調節持股，屬除息日特有的機械性賣壓，不宜全數讀為看空表態；區辨依據為9/17賣超是否收斂。⭐投信轉買166張(+166,543股)、自營商買超762張(自行買賣+64,300股→+64張、避險+697,916股→+698張，64+698=762與官方合計換算一致)；⭐全市場投信單日買超達NT$106.5億，是9/15賣超NT$19.9億的完全反轉。三大法人分項加總合計賣超7,816張(官方合計欄-7,815,621股換算-7,815，差1張屬正常捨入)。⚠️投信與自營合計買超928張僅能對沖外資賣超的10.6%。
+(5)⚠️⚠️技術面三項續惡化、一項持平，且惡化幅度有相當比例來自除息的機械缺口，本報逐項以「原始／還原除息」雙軌並陳：(a)⚠️MACD柱-13.00(還原後-12.11)，自-9.61續擴大、為連3日擴大；DIF自7.71急降至4.39、DEA自12.51降至10.89。⭐比負柱數值更值得追蹤的是DIF：自9/14的11.33在兩個交易日內降至4.39，即將下穿零軸，屆時代表12日與26日EMA正式交叉，屬中期趨勢轉折。(b)⚠️⚠️KDJ的J自-13.89再降至-17.25(還原後-15.88)，為連3日低於零軸且為本報追蹤期間最深；K自24.70降至17.75、D自44.00降至35.25。⭐成因可複算：9日窗口最高價仍為9/8的2,505、最低價因本日創低更新為2,375，RSV＝(2,380-2,375)÷(2,505-2,375)×100＝3.85。⚠️⚠️2,505將於9/21滾出9日窗口，屆時分母縮小、RSV會機械性回升，本報預先聲明屆時若無價格配合不會讀為動能改善。(c)⭐RSI原始值46.19、自46.88微降0.69點，⭐⭐但還原除息後為47.19、實為上升0.31點——本欄是本日唯一在雙軌下結論相反的指標，本報明確標示以避免誤導。(d)⚠️均線轉為四線失守：收2,380低於MA5 2,401、MA10 2,420、MA20 2,412、MA60 2,395；⭐僅MA120年線2,291仍在現價之下，現價高於年線89點(3.9%)。⭐布林通道續收斂：上軌2,471／中軌2,412／下軌2,352，帶寬自5.31%收窄至4.94%、為9/09(5.14%)以來最窄，⚠️惟仍寬於9/01至9/08的3.52%至4.70%、不是本波最窄。⭐技術指標口徑驗證：以同一套算法回算9/15已發布值(RSI 46.88／MACD柱-9.61／DIF 7.71／DEA 12.51／K 24.70／D 44.00／J -13.89／MA5 2,418／MA10 2,421／MA20 2,410／MA60 2,397／MA120 2,287／布林2,474-2,410-2,346／5日均量19,101)全數逐項完全複現，確認口徑未漂移。序列為TWSE官方2026-01-02至2026-09-16共171個交易日，⚠️該序列不還原除息。
+(6)⭐均線變化有一半以上與本日漲跌無關，須先剝除滾動窗口效應：(a)⭐⭐MA5自2,418大幅下滑17點至2,401，這17點100%來自窗口效應——滾出9/9的2,465、滾入2,380，(2,380-2,465)÷5恰為-17.0，與本日的除息與漲跌完全無關。(b)⭐MA10自2,421僅微降0.5點至2,420(滾出9/2的2,385)；⭐⭐MA20反而自2,410升1.5點至2,412(滾出8/19的2,350)、MA120自2,287升4.5點至2,291(滾出3/25的1,845)，即中長期均線仍在上彎、與MA5急墜方向相反，這是本報尚不宣告趨勢反轉的重要理由。(c)⚠️MA60季線自2,397降至2,395，收盤低於季線15點、較9/15的12點擴大；⭐但還原除息後的價差僅8點、實為收斂。⭐結論：跌破季線的狀態未解除，惡化程度被除息放大，實質上是沿季線下緣的橫向整理而非加速下跌，⚠️乾淨的判定時點是9/17。(d)⭐量能20,919張站上5日均量19,725張達6.1%、為9/08以來首見(9/09至9/15連5個交易日低於均量)，中止9/15因漢測凍資造成的量縮(漢測9/16上午抽籤、9/17解交股款，資金開始回流)；⚠️惟本日成交量含除息調節與月結算轉倉需求，不宜逕讀為買盤回流。全市場成交值回升至NT$6,759.70億(9/15為6,347.07億)。
+(7)⭐⭐期貨與選擇權(⚠️9/16為月結算日，所有未平倉皆為結清後重建的新基期，與9/15的比較在方向上完全沒有意義)：⭐合約更替聲明——台積電個股期CDF主力合約自202609換月至202610，舊合約202609於9/16為最後交易日、日盤收2,380、未平倉4,622口；新近月202610日盤收2,401(較前一交易日結算價+7)、成交6,831口、結算價2,401、未平倉25,169口。⚠️⚠️未平倉自9/15的7,291口跳升至25,169口(+245%)純粹是轉倉、不是新增部位，任何把它讀為多方大舉進場的敘述都是錯的。⭐基差：202610收2,401對現貨2,380為正價差21點(0.88%)，⚠️但其中約7點是機械性的——9月合約在9/16之前內含尚未發放的NT$7股利扣減、換月後該扣減消失，故相對9/15的+7點實質擴大約14點。⭐台指期TX 202610日盤收46,078(結算價46,060)、未平倉95,896口，對加權指數45,848.90為正價差229點。⭐TXO：買權未平倉37,215口、賣權31,098口、雙邊68,313口，較9/15的176,512口崩落61.3%(結算結清、非部位撤離)；P/C未平倉比83.56%(9/15為85.89%)，買權多於賣權、落在本報分段的「中性偏多」區間，⚠️惟結算當日比值可靠度遠低於平日。⭐成交量端出現典型結算特徵：買權352,656口、賣權375,087口、合計727,743口，較9/15的334,649口放大117.4%，成交量P/C比106.36%(9/15為106.44%、幾乎不變)——⚠️放量是結算平倉與轉倉造成、不是情緒升溫。⚠️本報既定日曆紀律：台指選擇權每週三與每週五都有到期結算，故P/C未平倉比只有在週一、週二、週四具備跨日可比性，9/17(週四)將是本次月結算後第一個可用的觀察點。⭐⭐⭐今晨夜盤(涵蓋FOMC宣布時點)：台積電個股期202610收2,422、較日盤收盤2,401大漲21點、量1,755口；台指期202610收46,382、較日盤收46,078上漲304點、量32,283口。⭐夜盤指示性在本報已有驗證紀錄(9/15夜盤2,387對現貨實收2,385僅差2點)，⚠️惟本次涵蓋FOMC、波動與指示性均高於平日，本報僅記錄不外推。
+(8)⭐評價：TWSE官方BWIBBU 9/16顯示P/E 27.59x、P/B 9.59x、殖利率0.92%(9/15為27.65x／9.61x／0.92%)，財報基準維持115/2未變動。⭐⭐本日評價下降百分之百來自除息：P/E降幅0.22%、P/B降幅0.21%，與股價因除息自2,385扣減至2,380的-0.21%幾乎完全相同，即分子(每股盈餘、每股淨值)未動、分母機械性下降，既非評價修正亦非財報基準換季。⚠️自9/16起本欄絕對水位相對9/15以前有約0.29%的向下位移，跨越9/16做評價比較請自行還原。⚠️BWIBBU殖利率採過去已發放股利計算，本次NT$7.00001要到10/8實際發放後才反映，短期內不會因本次除息跳升。市值約NT$61.7兆。ADR端P/E約30.8x、P/B約10.7x(依官方值×ADR溢價係數1.1152換算、非官方申報值)。⚠️百分位(P/E五年88%、十年89%、P/B五年92%)維持前值，單日0.2%變動不足以移動分位數。
+(9)⭐ADR溢價自10.06%擴大至11.52%(+1.46個百分點)，中止連續2日收斂：理論平價＝5×2,380÷31.77＝374.57(採捨入後匯率)，對市價417.72之溢價+11.52%；台股端因除息機械扣減-0.21%(分母降)、ADR端+0.96%(分子升)，兩者反向必然推升溢價。⭐⭐本日有一項罕見的有利條件：台股2330與ADR TSM於9/16「同日」除息(台股NT$7.00001、ADR依Yahoo股利事件記錄為每單位US$1.107毛額)，故分子與分母同步扣減，本欄未受一般常見的除息時間差污染、可與9/15直接比較。⭐⭐附帶解決一項本報長期懸而未決的疑問：stockanalysis.com以還原股利後的前收412.88計算9/16漲幅為+1.17%，而原始價漲幅為+0.96%，兩者差額0.21個百分點即ADR端的股利效果，由此反推ADR每單位淨股利約US$0.87；與台股NT$35.00(7.00001×5)÷31.77＝US$1.10的毛額相比，隱含約21%的台灣股利扣繳率，與現行稅制相符——即US$1.107至1.114為毛額、US$0.87為投資人實收淨額，兩者並不矛盾。⭐相對強弱：近5日-3.45%(基準9/9收2,465、未還原除息，還原後-3.16%)，大盤近5日-2.83%；近1月-0.63%(基準8/14收2,395，還原後-0.33%)，大盤+0.08%；YTD+50.2%(基準2026-01-02收1,585；2026年以來三次除息合計NT$19.000073，還原後約+51.4%)，落後大盤+56.2%與費半+52.7%。⚠️本日台股2330 +0.08%明顯落後加權指數+0.74%，且加權指數本身含反向機械成分——媒體統計台積電等3檔個股9/16除息合計使指數減少56.59點，還原後加權指數實為+0.86%，台積電落後幅度比字面更大；⭐但台積電ADR +0.96%是領先費半+0.63%的，台美兩端方向相反，列為明日觀察項。
+(10)⚠️匯率9/11起連4日走貶：新台幣9/16交易日收31.7734(本報採31.77)，較9/15的31.7176再貶0.18%，自9/10的31.4640累計貶值0.98%，對毛利率影響約+39bps、已升級為對單季毛利率具實質貢獻。⚠️口徑更正：前一份日報敘述為「連續第4個交易日、四日累計自31.464」，本報回頭核對後確認31.464對應9/10當日值、而9/10相對9/09的31.4992是升值，故自本日起改採「9/11起連續4日、基準31.4640」的寫法，數值無誤、僅計數起點更精確。⚠️取數限制：本欄採Yahoo TWD=X日K棒收盤而非銀行間16:00定盤價。⭐今晨9/17台北09:16前後盤中報31.875，較9/16收盤再貶0.32%，屬盤中值不納入計算。⭐附帶驗證：前一份日報所記「9/16今晨盤中31.851」與本日確認的9/16正式收盤31.7734相比高估0.08，顯示盤中值與收盤值差距可達0.25%，本報維持不以盤中值入帳的作法正確。
+(11)⭐供應鏈與客戶端19檔追蹤標的13漲6跌，分布證實「升息未壓抑半導體、但族群內部高度分化」：⭐漲幅前段為華邦電+5.96%收169.00元(中止連5日下跌、為本日漲幅最大者)、SK海力士+4.08%收1,759,000韓元(為9/11以來最高收盤，惟三日累計仍-2.92%)、Intel+4.03%收$101.05(收復$100、量1.19億股為9/11以來最高)、聯發科+2.26%收4,530元、日月光+2.20%收605.00元(收復600元)、三星+2.01%收253,500韓元——⭐⭐前六名中五名為亞洲掛牌標的(僅Intel為美股)、其中兩名為記憶體，顯示買盤集中在亞股補漲與記憶體而非美系設備或AI伺服器鏈。⚠️跌幅端共6檔：高通-1.58%收$184.84(為本日跌幅最大，屬吐回9/15大漲的一部分、三日累計仍+1.58%)、應材-1.38%收$415.38(連3日黑、三日累計-9.01%、再創本波新低)、科林-0.61%收$269.23(三日-9.72%、為全部標的中三日跌幅第二深)、科磊-0.39%收$167.36、Amkor-0.22%收$46.28(連3日黑、三日-10.54%為全部標的中三日跌幅最深)、美光-0.11%收$926.55(在亞洲記憶體大漲的一天無反應)。⭐設備四雄三跌一漲、艾司摩爾+0.67%收$1,602.22為唯一收紅。⭐蘋果+0.32%收$332.41、三日累計+0.04%，與高通+1.58%同為19檔中僅有的兩檔三日正報酬。⭐輝達+0.82%收$213.90，與台積電ADR +0.96%方向一致且幅度相近，與9/15的方向相反明確不同。
+(12)⭐台積電相關事件三則：(a)⭐⭐聯發科發表天璣9600 Pro採用台積電2奈米(N2)製程，神經處理器在生成式AI首次提示處理效能較前代提升51%；同系列9600M維持3奈米。⭐意義在於N2放量客戶擴增——依台積電2026年第2季數據，2奈米僅占晶圓營收3%、3奈米30%、5奈米33%，每增加一家N2量產客戶都是後續營收結構的實質增量，且N2的ASP高於N3。⚠️本報未取得該晶片量產時程與投片量，無法量化單季貢獻(來源Yahoo Finance，2026-09-17)。(b)⭐博通執行長Hock Tan公開預估該公司AI相關營收2028年可達2,300億美元，對台積電先進製程與CoWoS的訂單能見度延伸至2028年；⚠️屬單一企業長期展望而非已簽訂單，且博通股價9/16僅+0.07%、三日累計-6.21%，市場尚未定價。(c)⭐超微、博通、Meta、微軟、輝達與OpenAI共組Optical Scale-up Consortium，為AI基礎設施制定開放式光互連規格，對台積電屬間接利多(矽光子與共同封裝光學均須先進封裝支援)；⚠️該聯盟成立確切日期未能證實、僅確認出現於9/16報導中，且無量化採購承諾，列為長期觀察項。⚠️另有彙整報導稱中國中芯與長鑫存儲DRAM市佔推進至約10%，原始出處未逐一驗證，本報列為待證實的中長期競爭觀察項、不納入當期判斷。
+(13)⭐除息與股利完整資訊：本次為台積電首度季配息達7元，現金發放日2026-10-08。⭐⭐下一次除息日為2026-12-10(第2季季配息，8/11董事會拍板續配NT$7.00)，現金發放日2027-01-07；⭐該次起外資股東首度可選擇以美元領取股息。⭐本報已於本日重新以TWT48U查詢2026-09-01至2026-10-31全區間，確認該區間內2330僅9/16一筆除息、無遺漏(本報自2026-09-10起將除息預告列為每週至少查核一次的獨立項目)。⭐2026年以來三次除息合計NT$19.000073(3/17的6.000036、6/11的6.000036、9/16的7.000001，Yahoo股利事件序列確認)。
+(14)⭐⭐明日(9/17)五項檢核，將逐條回頭驗證：(a)第一順位「次日填息能否完成」——今晨09:05台北時間盤中已報2,415、高於除息前收盤2,385達30元，若收盤守在2,385之上即完成次日填息，本報將把9/16的失敗改判為單日雜訊；⚠️反之若收盤跌回2,385之下，連續兩日填息失敗須視為需求面的實質警訊。(b)第二順位「外資賣超是否隨除息日結束而收斂」——若收斂至3,000張以下則歸因於除息；若維持8,000張以上則須升級為趨勢性撤出並下調本報立場。(c)第三順位「MACD與KDJ的背離是否解除」——今日起除息缺口不再干擾比較、是乾淨的判定時點：若價站穩2,400之上而負柱自-13.00開始收斂則背離解除。(d)第四順位「升息後的半導體定價」——觀察費半能否連3日收紅。(e)第五順位「衍生品新基期的首個可讀訊號」——9/17(週四)是本次月結算後第一個具跨日可比性的P/C未平倉讀數。⚠️本報立場維持「中性偏空」不變，理由是三項偏空(當日填息失敗、外資賣超擴大且單檔輪出連2日、MACD與KDJ連3日惡化且J值創追蹤期間最深)與三項偏多(升息落地而半導體不跌反漲、今晨夜盤個股期大漲21點且台股實際開高至2,415、量能回升至5日均量之上且2,375前低首度受測即守住)恰好抵銷。⚠️⚠️本報明確不因今晨開高而預先轉為中性——既定紀律為只用已收盤數據定調，今晨的2,415屬盤中值，且9/15的止跌訊號在9/16已被證明未能延續，同一錯誤不重犯第二次。⚠️須誠實聲明：「中性偏空」是對未來1至5個交易日技術面與籌碼面的判斷，不含對台積電基本面的負面看法——8月營收創新高、連11季超預期、聯發科N2新單、Q3法說會預計10月中旬，這些基本面事實在本輪修正中沒有任何一項改變。</t>
+        </is>
+      </c>
+      <c r="G128" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:G2"/>

</xml_diff>

<commit_message>
daily: 2026-09-18 日報 HTML & Excel 更新
資料日 2026-09-17：台股 2330 收 2,425（+45、+1.89%），開盤即完成 9/16 除息的
填息；外資自連 5 日賣超反手買超 4,794 張；ADR 收 $430.26（+3.00%）、費半
+3.14% 連三日反彈；今晨夜盤台指期 +701 點。

驗證：TWSE STOCK_DAY／BWIBBU／T86／BFI82U／FMTQIK 與 TAIFEX 均自官方端點取數；
ADR 與美股收盤經 stockanalysis.com 與 investing.com 雙來源交叉確認；技術指標
以前一交易日 replay 全項複現 9/16 已發布值。

本次另更正 13 處排名／極值與期間報酬敘述（經 fresh-context 驗收與自行複算）：
均線「首度站上五條」改為「9/09 以來首見」、P/C 可查交易日 23→22、MACD「本波
最大」改為「9/14 轉負以來首次收斂」、費半與三大法人的「9 月以來最大」改為明確
基準日、生態系 4 檔「三日累計」基準日統一為 9/14，並為各項極值敘述加註核算範圍。

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -912,7 +912,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-09-17</t>
+          <t>報告更新日期：2026-09-18</t>
         </is>
       </c>
     </row>
@@ -3377,7 +3377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G128"/>
+  <dimension ref="A1:G129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3399,7 +3399,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-09-17</t>
+          <t>最後更新：2026-09-18</t>
         </is>
       </c>
     </row>
@@ -8156,6 +8156,58 @@
         </is>
       </c>
     </row>
+    <row r="129">
+      <c r="A129" s="50" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B129" s="50" t="inlineStr">
+        <is>
+          <t>NT$2,425（9/17收，填息完成）</t>
+        </is>
+      </c>
+      <c r="C129" s="51" t="inlineStr">
+        <is>
+          <t>+1.89%（9/17收，+45.00）</t>
+        </is>
+      </c>
+      <c r="D129" s="50" t="inlineStr">
+        <is>
+          <t>US$430.26（9/17收，+3.00%）</t>
+        </is>
+      </c>
+      <c r="E129" s="50" t="inlineStr">
+        <is>
+          <t>18,117（9/17收）</t>
+        </is>
+      </c>
+      <c r="F129" s="52" t="inlineStr">
+        <is>
+          <t>報告日2026-09-18(Fri)，台股資料為2026-09-17(Thu)官方收盤；ADR、費半與全部美股個股為9/17美東收盤(台北9/18清晨)；期貨含今晨夜盤(TAIFEX標記9/18之盤後列，實際時段9/17 15:00至9/18 05:00)。
+(0)⚠️三項閱讀前提：(a)9/16為除息日(每股NT$7.00001、除息參考價2,377.99、除息前收盤2,385.00)，本行台股價格自9/16起為未還原原始價，跨越9/16與9/15以前比較須自行還原。(b)9/16為9月台指期與選擇權月結算日，個股期主力合約已自202609換月至202610，本行期貨數字為新合約、不可與202609跨合約比較。(c)今日9/18為週五、台指選擇權有週結算，本行所載未平倉與P/C比將於當日重置。
+(1)⭐⭐⭐本日最重要的事是填息完成，且前一份日報的第一順位檢核據以通過：台股2330官方收NT$2,425(開2,405／高2,445／低2,400／量18,117張、額NT$439.33億、61,567筆，TWSE STOCK_DAY確認)，漲跌價差欄恢復正常揭示為+45.00(對9/16收盤2,380、+1.89%)。⭐開盤2,405即已高於除息前收盤2,385達20元，全日最低2,400不曾失守填息價，收2,425高出2,385達40元——即不僅完全填息、還在填息之上再漲1.68%。⭐前報曾言「若收盤守在2,385之上即完成次日填息，本報將把9/16的失敗改判為單日雜訊」，本報依約執行此改判；台積電近5次除息全數於兩個交易日內填息的紀錄獲得延續。⚠️惟須並陳一項保留：收盤2,425距當日高點2,445仍有20元，尾盤有獲利了結壓力，非全日一路走高。
+(2)⭐⭐逐條履行前一份日報所訂四項檢核，結果為三項通過、一項未通過：(a)第一順位「次日填息能否完成」——通過，理由見(1)，且為強度最高的一種通過方式(開盤即完成、全日未回測)。(b)第二順位「MACD負柱是否續擴大至-13以上」——未擴大、反而收斂至-8.90，為連3日擴大後首度收斂；⭐前報當時以還原除息對照組僅-12.11為由判定9/16的-13.00「字面成立、實質未成立」並拒絕追認反彈失敗，本日的收斂事後證明該項保留是正確的，本報記錄此點以供日後校準判斷尺度。(c)第三順位「夜盤指示能否兌現」——通過：前報所記今晨個股期202610收2,422與09:05盤中報2,415，本日正式收盤2,425高於兩者。(d)⚠️第四順位「量能能否站回均量之上」——未通過，理由見(6)，本報將此項延續為次日第一順位檢核。
+(3)⭐⭐⭐籌碼面本日出現本報追蹤期間罕見的完全反轉，且須用三個層次才說得完整：(a)外資對台積電單日買超4,794張(TWSE T86官方買進13,315,712股／賣出8,521,522股／淨+4,794,190股，依既定口徑向零截斷)，以2,425元計約NT$116.3億，中止自9/10起連續5個交易日的賣超，單日方向擺盪達13,538張。(b)⭐⭐全市場層面同向印證且與9/16形成關鍵對照：TWSE BFI82U顯示9/17全市場外資淨買超NT$121.85億、投信NT$117.03億、自營商NT$15.78億、三大法人合計NT$254.66億；⭐9/16台積電單檔賣超金額曾「超過」全市場外資淨賣超總額(資金自台積電輪出至其他台股)，而本日台積電單檔買超NT$116.3億占全市場外資淨買超NT$121.85億的95.4%，即外資本日買盤幾乎全數集中於台積電一檔，輪出結構已反轉為輪入。(c)⚠️惟一項未同步的證據須並陳：投信對台積電本日反而小幅賣超59張(-59,590股)，與全市場投信大買NT$117.03億方向相反，即投信買盤流向台積電以外標的。⭐自營商買超509張(+509,161股)為連續第4日買超，分項自行買賣+356,900股(+356張)、避險+152,261股(+152張)，兩者向零截斷後相加508張與官方合計換算值509張差1張屬正常捨入。⭐三大法人依分項加總合計淨買超5,244張(官方合計欄+5,243,761股)，為9/08(當時6,303張)以來單日最大淨買超。
+(4)⭐⭐技術面四項指標全數由惡化轉為修復：(a)MACD柱自-13.00收斂至-8.90(收斂幅度4.10為負柱自9/14轉負以來的首次收斂(9/14至9/16三日均為擴大))、為連3日擴大後首度收斂；DIF自4.39回升至5.32、DEA自10.89降至9.78，兩者差距自-6.50收斂至-4.45。⚠️但尚未轉正——DIF仍在DEA之下4.45、黃金交叉未發生，本報不以單日收斂逕自宣告轉強。(b)⭐⭐KDJ的J自-17.25(本報追蹤期間最深)單日大幅回升27.78點至+10.53、重返零軸之上，中止連3日負值；K自17.75升至24.65、D自35.25降至31.72，K與D的負乖離自-17.50收斂至-7.07，⚠️惟KD黃金交叉亦尚未發生。⭐成因可複算：9日窗口最高2,505(9/08)、最低2,375(9/16)，本日收2,425的RSV＝(2,425-2,375)÷(2,505-2,375)×100＝38.46，較9/16的3.85大幅墊高。(c)RSI 14自46.19升6.66點至52.85、重返50中軸之上，為9/10以來首見。(d)⚠️唯一未改善者為布林帶寬：自4.94%續收窄至4.75%，上軌2,472／中軌2,414／下軌2,357。⭐口徑驗證：以同一套算法回算9/16已發布值(RSI 46.19／MACD柱-13.00／DIF 4.39／DEA 10.89／K 17.75／D 35.25／J -17.25／MA5 2,401／MA10 2,420／MA20 2,412／MA60 2,395／MA120 2,291／布林2,471-2,412-2,352／5日均量19,725)全數逐項完全複現，確認口徑未漂移。序列為TWSE官方2026-01-02至2026-09-17共172個交易日、不還原除息，另備還原除息對照組(9/16起加回NT$7.00001)交叉檢核，本日原始與還原兩組結論方向全部一致(還原組為RSI 53.78／MACD柱-7.50／K 26.09／D 32.32／J 13.62)。
+(5)⭐⭐均線本日出現本報追蹤期間第一次「現價同時站上全部五條均線」，空頭排列的成形過程中止：MA5 2,396／MA10 2,424／MA20 2,414／MA60 2,396／MA120 2,296，收盤2,425全部站上。⚠️但其中最醒目的一項變化必須先剝除機械成因：MA5在股價大漲45元的一天反而自2,401「下降」5點至2,396——這100%來自滾動窗口效應，可逐點複算：滾出9/10的2,450、滾入2,425，(2,425-2,450)÷5恰為-5.0，與本日漲跌完全無關；「股價大漲而5日線下降」在直覺上矛盾、極易被誤讀為背離，本報特別標示。⭐其餘四線同步上行：MA20自2,412升至2,414(滾出8/20的2,375，(2,425-2,375)÷20＝+2.5)、MA10自2,420升至2,424、MA60自2,395升至2,396、MA120自2,291升至2,296。⭐現價與各線的距離決定明日的脆弱程度：高於MA10僅1元(五條中最接近、最易失守)、高於MA20有11元、高於MA5與MA60各29元、高於MA120有129元。
+(6)⚠️⚠️本日唯一與價格方向背離、且必須誠實指出的欄位是量能：成交18,117張較9/16的20,919張減少13.4%，且低於本報所計5日均量19,381張達6.5%，即本日上漲屬「價漲量縮」。⭐惟須並陳一項可查證的成因：9/16的20,919張本身含除息與月結算的被動調節與轉倉成交、並非乾淨的自然量；若改與9/15的15,216張(無事件干擾日)相比，本日為增加19.1%。⭐本報結論是「量能不足以追認為趨勢突破，但亦非量能萎縮」，並因此僅將立場自「中性偏空」上調一級至「中性」而非直接轉為偏多。
+(7)⭐期貨與選擇權：⭐台積電個股期CDF 202610日盤收2,433(+32點)、結算價2,432、未平倉25,045口(自9/16的25,169口微減124口)，對現貨2,425的基差+8點正價差、較9/16的+21點收斂，⭐基差收斂而未轉負屬期現同步上漲下的正常現象。⭐台指期TX 202610日盤收46,445(+385)、結算價46,459、未平倉99,476口。⭐⭐⭐今晨夜盤(9/17 15:00至9/18 05:00、涵蓋美股9/17全場)：台積電個股期202610收2,459、較日盤結算價2,432大漲27點、量1,232口；台指期202610收47,160、較日盤結算價46,459大漲701點、量21,169口——⚠️該701點為 9 月以來 14 個夜盤中最大的單場漲點（本報已抓 TAIFEX 9/01 至 9/18 全部夜盤排序確認，次大為 9/04 的 +668 點；⚠️ 本報僅就 9 月此一已核算區間陳述，不宣稱更長期間的紀錄），指向今日台股開盤可能明顯跳空；⚠️夜盤只指示開盤方向、不指示收盤。⭐TXO：買權未平倉76,415口、賣權58,457口、雙邊134,872口，P/C未平倉比76.50%，⭐為TAIFEX pcRatioDown目前可查的22個交易日(2026-08-19至09-17)中最低值，本報已將該區間全部22筆排序確認、未超出可查範圍作更長期宣稱；買權未平倉多於賣權達31%、結構上偏多。⚠️⚠️可比性有兩項限制：9/16為月結算日、9/17是重建後第一個交易日屬新基期，與9/16的83.56%作方向性比較意義有限；且今日9/18週五另有週結算、未平倉將再次重置，故本日的偏多結構不具延續至下週的可比性。⚠️外資台指期多空未平倉淨額為-78,674口(多8,161／空86,835)、較9/16的-76,351口再擴大2,323口淨空單——與現貨端大買台積電方向相反，是本日唯一的內部矛盾訊號，可能為避險亦可能為對大盤的方向性看空，本報無法由公開數據區分，列為待觀察而不作歸因。
+(8)⭐評價：TWSE官方BWIBBU 9/17顯示P/E 28.11x、P/B 9.78x、殖利率0.91%(9/16為27.59x／9.59x／0.92%)，財報基準維持115/2未變動。⭐⭐本日評價上升百分之百來自股價：P/E升幅1.88%、P/B升幅1.98%，與股價漲幅+1.89%一致，即分子(股價)動、分母(獲利與淨值)未動，非獲利預期重估。⚠️續提醒：8月營收雖於9/10創歷史新高，但官方P/E採115Q2基準，月營收要到Q3財報認列後才反映在分母，若Q3如預期成長，換季當日P/E將出現一次性下修(參照8/14自115Q1換至115Q2時P/E由32.74x一次降至27.76x的前例)。市值約NT$62.9兆。ADR端P/E約31.8x、P/B約11.1x(依官方值×ADR溢價係數1.1306換算、非官方申報值)。
+(9)⭐ADR TSM 9/17正式收盤$430.26(+$12.54、+3.00%)，已用stockanalysis.com與investing.com雙獨立來源交叉確認(兩來源收盤價、漲跌額、前收皆完全一致)，並通過「前收417.72×(1+3.00%)＝430.25≈430.26」自我檢核；⭐本日兩來源前收皆為未還原的417.72、不存在9/16那種還原股利口徑差異。⭐+3.00%為ADR自9/08以來最大單日漲幅、明顯強於台股同日的+1.89%，兩市差距1.11個百分點。⭐ADR溢價自+11.52%擴大至+13.06%(連續第2日擴大)：理論平價＝5×2,425÷31.86＝380.57(採捨入後匯率)，對市價430.26之溢價+13.06%；成因是兩項同向因素疊加——ADR漲幅大於台股(分子增幅大於分母)，且新台幣同步走貶(平價分母再降)。⭐相對強弱：近5日-1.02%(基準9/10收2,450)、大盤-1.39%；近1月+1.04%(基準8/17收2,400，⚠️該基準採日曆同日、每日移動)；YTD+53.0%(基準2026-01-02收1,585)，大盤+57.7%、費半+57.4%。⭐本日台股2330 +1.89%明顯領先加權指數+0.96%(收46,288.00、+439.10)，與9/16的落後完全相反。
+(10)⚠️匯率9/11起連5日走貶：新台幣9/17收31.8596(本報採31.86)，較9/16的31.7734再貶0.27%，自9/10的31.4640累計貶值1.26%，依本報敏感度表約對應毛利率+50bps的換算助益。⭐方向對台積電以美元計價營收換算有利，⚠️惟為換算效果而非需求改善，不應與訂單面利多混為一談。⭐交叉驗證：台灣銀行9/17牌告即期買入31.83／賣出31.93(中價31.88)，與本報採用的Yahoo中間價31.8596相差0.02、差異來自銀行買賣價差，兩者可互相印證。⚠️取數限制同前：本欄採Yahoo TWD=X日K棒收盤而非銀行間16:00定盤價。
+(11)⭐供應鏈與客戶端19檔追蹤標的16漲3跌，且分歧的軸線是「交易時區」而非產業次族群：⭐⭐漲幅前段Arm+8.57%收$264.90(為19檔中漲幅最大、三日累計轉為+10.83%)、Intel+7.67%收$108.80(兩日累計+12.01%)、超微+6.36%收$545.09(三日+10.47%、外電以「AMD領漲」為標題)、美光+5.50%收$977.50(9/16在亞洲記憶體大漲時-0.11%毫無反應、本日反過來領漲)、Amkor+3.61%收$47.95(中止連3日下跌)、費半+3.14%收11,599.49——全部為美股。⚠️而3檔下跌者為SK海力士-0.80%收1,745,000韓元、聯發科-0.66%收4,500元、三星-0.39%收252,500韓元——全部為亞洲掛牌標的，成因單純且可查證：亞洲9/17盤在美股9/17大漲之前就已收盤、尚未反映該波漲勢。⭐今晨韓股盤中SK海力士報1,825,000韓元(+4.58%)、三星報259,000韓元(+2.57%)，兩者皆已大幅補漲，⚠️此為台北時間08:56的盤中價、非收盤價，次一份日報將以正式收盤價回頭補正。⭐設備四雄本日全數收紅為9/11以來首次一致收紅(艾司摩爾+1.71%、科磊+0.97%、應材+0.49%、科林+0.03%)，⚠️惟四檔漲幅全部低於費半的+3.14%，即本輪反彈的資金並未流向設備股，本報續列設備股為AI資本支出的前導觀察指標。⭐輝達+2.54%收$219.34、蘋果+1.38%收$337.00(創本波新高、逼近52週高$344.57)、博通+2.29%收$347.30、高通+2.09%收$188.71。
+(12)⭐美股總體9/17全面轉為風險偏好：標普500收7,637.76(+1.14%)、那斯達克26,418.30(+1.69%)、VIX自17.71大跌12.82%至15.44。⭐⭐本日最值得記錄之處在於它推翻了一項合理的擔憂：聯準會9/16升息1碼至3.75-4.00%(2023年以來首次、12比0一致決)之後，半導體不僅未被壓抑，反而在次日連三日走強。⚠️惟據CNBC報導18位官員中有16位預期年內再升一次，主席Kevin Warsh指通膨「過高且持續過久」、中東情勢推升油價為本次升息主因；若該升息路徑被後續官員談話確認，本波把升息定價為「一次性事件」的前提存在被推翻的風險。⭐外電(24/7 Wall St，2026-09-17)指出當日QQQ漲幅明顯小於費半，即買盤高度集中於半導體而非科技股全面回升，並將主因歸於AI資本支出與需求面帶動的類股輪動、而非單一總經事件。
+(13)⭐台積電相關事件兩則：(a)⭐聯發科9/15發表天璣9600 Pro採用台積電2奈米製程、內含33億顆電晶體，外電報導多核心功耗較前代降低61%、單核效能提升17%，為業界首款量產的2奈米手機晶片，vivo X500系列預定9/21首發搭載(來源9to5Google，2026-09-15)。⚠️須標註一項未能證實之處：關於該晶片究係採用N2或N2P製程，不同來源說法不一，本報未取得台積電或聯發科官方確認。(b)⭐外電報導台積電2026年底CoWoS月產能目標上修至約12.5萬片、較2025年底增20-30%，新增產能開出前已被輝達(逾五成)與博通預訂一空(來源TechNews，2026-09-12)。⚠️本報須並陳一項口徑差異、不逕自合併引用：本報CoWoS區塊所載2026年目標約35,000 wspm來自TrendForce 2026-Q1預估，與本則的12.5萬片係不同來源與不同計算基礎，兩者不可直接相減或並列，本報未取得台積電官方產能數字以資調和，標示為未能證實。⭐8月營收NT$5,148.1億(+53.3% YoY、+10.1% MoM)、前八月累計約NT$3.3869兆(+39.3% YoY)於9/17的類股反彈中仍被外電反覆引用為AI需求未見頂的核心證據。
+(14)⭐⭐明日(9/18本報告日)五項檢核，次一份日報將逐條回頭驗證：(a)⚠️⚠️第一順位「量能能否站回5日均量19,381張之上」——9/17的上漲是價漲量縮，本報正因此項而僅上調至中性、未直接轉多；若量能站回均量之上且收盤守穩，將把9/17的上漲追認為趨勢突破，反之維持中性。(b)⭐⭐第二順位「夜盤指示能否再度兌現」——今晨台指期夜盤大漲701點、個股期收2,459，指向明顯跳空開高；⚠️夜盤只指示開盤不指示收盤，具體檢核是「收盤能否守在2,445(9/17盤中高)之上」。(c)第三順位「外資買超能否連續」——9/17的買超屬單日反轉，須至少連續2日才構成趨勢。(d)第四順位「兩項黃金交叉能否成立」——MACD的DIF 5.32仍在DEA 9.78之下4.45、KDJ的K 24.65仍在D 31.72之下7.07，兩項皆未發生。(e)⚠️第五順位「週結算後的未平倉重置」——今日為週五、台指選擇權有週結算，次一份日報引用未平倉與P/C比時須標註重置效應。⚠️⚠️本報立場自「中性偏空」上調一級至「中性」，理由是四項偏多(填息完成且開盤即達成、外資反手買超且占全市場95.4%、技術面四項同步修復、收盤恢復站上全部五條均線（9/09 以來首見）)對一項偏空(價漲量縮、量能低於均量6.5%)；⭐本報明確不因單日大漲而直接轉為偏多——既定紀律是量價須同步確認，且9/15的止跌訊號在9/16已被證明未能延續，同一錯誤不重犯第二次。⚠️須誠實聲明：本報立場是對未來1至5個交易日技術面與籌碼面的判斷，不含對台積電基本面的負面看法。</t>
+        </is>
+      </c>
+      <c r="G129" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:G2"/>

</xml_diff>

<commit_message>
daily: 2026-09-21 日報 HTML & Excel 更新
涵蓋 2026-09-18(Fri) 收盤：台股 2330 收 2,460 (+35.00/+1.44%)、量 40,893 張；
ADR TSM 收 434.67 (+1.03%)。

主要判斷：9/18 爆量含 FTSE TWSE 台灣指數系列季度審核生效日的被動調節成分
(對照組權值股同步爆量、全市場股數僅 +12.5%、筆數 +13.0% vs 股數 +125.7%)，
故前報第一順位量能檢核判為「字面通過但拒絕追認為趨勢突破」；立場自中性上調至中性偏多。

自查修正三項過度宣稱：
- 三大法人合計 7,878 張非追蹤期間最大 (7/01 以來 57 日中排第 5)，改為「9/07 以來最大」
- 成交量 40,893 張非極端值 (2026 年 173 日中排第 65)，改為區分「單日增幅」與「絕對水位」
- 外資台指期淨空單收斂改標明核算範圍僅及 9/16 起

另訂正 52 週低點滾動窗口失效值 (台股 1,265→1,270、ADR 257.98→265.45)，
並以正式收盤價回補前報所引韓股盤中價 (SK 海力士 1,857,000/+6.42%、三星 261,000/+3.37%)。

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -912,7 +912,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-09-18</t>
+          <t>報告更新日期：2026-09-21</t>
         </is>
       </c>
     </row>
@@ -3377,7 +3377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G129"/>
+  <dimension ref="A1:G130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3399,7 +3399,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-09-18</t>
+          <t>最後更新：2026-09-21</t>
         </is>
       </c>
     </row>
@@ -8208,6 +8208,54 @@
         </is>
       </c>
     </row>
+    <row r="130">
+      <c r="A130" s="53" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B130" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,460（9/18收，爆量40,893張含指數調節）</t>
+        </is>
+      </c>
+      <c r="C130" s="54" t="inlineStr">
+        <is>
+          <t>+1.44%（9/18收，+35.00，落後大盤+1.93%）</t>
+        </is>
+      </c>
+      <c r="D130" s="53" t="inlineStr">
+        <is>
+          <t>US$434.67（9/18收，+1.03%）</t>
+        </is>
+      </c>
+      <c r="E130" s="53" t="inlineStr">
+        <is>
+          <t>40,893（9/18收，+125.7%）</t>
+        </is>
+      </c>
+      <c r="F130" s="55" t="inlineStr">
+        <is>
+          <t>報告日2026-09-21(Mon)，台股資料為2026-09-18(Fri)官方收盤；ADR、費半與全部美股個股、韓股為9/18正式收盤；期貨為TAIFEX 9/18日盤，另含9/18夜盤(9/18 15:00至9/19約05:00、涵蓋美股9/18全場)。
+(0)⚠️三項閱讀前提：(a)9/19與9/20為週末，今晨(週一)並無夜盤場次，本行所引夜盤為9/18週五晚間那一場，與今日開盤之間隔了整個週末，指示性弱於平日。(b)9/18為台指選擇權週結算日，本行所載TXO未平倉與P/C比為結算後的新基期讀數，與9/17不具可比性。(c)本行新台幣匯率採Yahoo TWD=X序列經台北時區換算後之當日值31.8511，與前一行同一口徑故可比；另有在岸收盤31.808之說，差異與影響見(8)。
+(1)⚠️⚠️本日最重要的事是成交量暴增的性質，且本報的結論是「不可照字面採信」：台股2330官方收NT$2,460(開2,460／高2,460／低2,435，開＝高＝收；量40,893張、額NT$1,003.94億、69,571筆，TWSE STOCK_DAY確認)，漲跌價差+35.00(對9/17收盤2,425、+1.44%)。⭐前一份日報列為第一順位檢核的「量能能否站回5日均量19,381張之上」，字面上以40,893張大幅通過(超出111%)。⚠️⚠️但本報拒絕據此把9/17-9/18的上漲追認為趨勢突破，三項可查證依據：(a)事件面——9/18為FTSE TWSE台灣指數系列(含台灣50，0050規模約NT$2.35兆)季度定期審核生效日，FTSE Russell通知id=2621873載明effective after the close of business on Friday, 18 September 2026，該日亦為九月第三個週五(全球季度再平衡與四巫日)。(b)對照組——TWSE MI_INDEX實抓9/17→9/18成交股數倍數：日月光投控2.49x、台積電2.26x、國泰金2.22x、富邦金2.01x、中華電1.84x、鴻海1.69x、聯發科1.60x、台達電1.21x、聯電1.19x、台塑1.12x，而全市場成交股數僅自10,710,347,398增至12,052,158,761(+12.5%)；即爆量集中於指數成分股而非全市場普遍放量，且台積電的2.26x在樣本中並非最高，故非台積電特有事件。(c)型態面——成交筆數僅自61,567增至69,571(+13.0%)而成交股數增125.7%，平均每筆張數大增屬大單特徵；且開＝高＝收＝2,460，收盤精準落在全日最高點，與被動資金於收盤集合競價一次性調節部位的型態吻合。⚠️本報未能取得FTSE官方附件中2330自身權重調整幅度(Excel附件未能解析)，故無法量化機械成分的確切比例，明確標示為未能證實、不編造比例。
+(2)⚠️⚠️與爆量並列、同樣不利於樂觀解讀的一項事實是相對弱勢：台積電+1.44%落後同日加權指數+1.93%(TWSE FMTQIK官方46,288.00→47,180.75、+892.75點)達0.49個百分點；⭐由於台積電占加權指數權重約三成，指數漲幅高於台積電意味著非台積電成分股的平均漲幅明顯更高。同屬台系半導體者全數跑贏：聯發科+4.67%(收4,710)、華邦電+5.59%(收179.5)、日月光投控+3.91%(收638)。ADR端同樣落後：TSM+1.03%，而同日費半+2.78%、應用材料+6.51%、科林研發+6.98%。⭐此與「爆量來自被動調節而非主動追價」的判讀互相一致。
+(3)⭐⭐逐條履行前一份日報所訂四項檢核，結果為三項通過、一項字面通過但實質存疑：(a)⚠️⚠️第一順位「量能能否站回5日均量19,381張之上」——字面通過但本報拒絕追認為趨勢突破，理由見(1)。(b)⭐第二順位「夜盤指示能否再度兌現」——通過：前報所記9/17夜盤台指期大漲701點指向開高，9/18果然跳空高開35元至2,460。(c)⭐第三順位「外資台指期淨空單是否續擴大」——未擴大反收斂：9/18外資臺股期貨多空未平倉淨額-76,110口(多10,323／空86,433)，較9/17的-78,674口減少2,564口淨空單，為本報自 9/16 起逐日記錄此項以來的首見收斂（⚠️ 本報的核算範圍僅及於 9/16 起的數個交易日，不宣稱更長期間）。(d)⭐第四順位「亞洲標的補漲須以正式收盤價回頭補正」——已補正：SK海力士9/18正式收盤1,857,000韓元(+6.42%)、三星電子261,000韓元(+3.37%)，⭐兩者實際漲幅皆大於前報所引台北時間08:56的盤中價(1,825,000／+4.58%、259,000／+2.57%)，前報的保留方向正確惟幅度被低估。
+(4)⭐⭐籌碼面維持買超但結構由集中轉為分散：(a)外資對台積電買超6,039張(TWSE T86官方買進32,975,037股／賣出26,935,685股／淨+6,039,352股，依既定口徑向零截斷)，以2,460元計約NT$148.57億，為連續第2個交易日買超、兩日合計10,833張。(b)⚠️惟集中度大幅下降：TWSE BFI82U顯示9/18全市場外資淨買超NT$869.94億，台積電單檔NT$148.57億僅占17.1%——⭐與9/17的95.4%形成強烈對照，即外資9/17幾乎全壓台積電一檔、9/18則轉為全面撒網，與指數審核生效日須同時調整多檔成分股的特性一致。(c)投信由賣轉買478張(+478,401股)、自營商買超1,361張(+1,361,432股)為連續第5日買超；⚠️自營商分項自行買賣+978,545股(+978張)、避險+382,887股(+382張)，向零截斷後相加1,360張與官方合計換算值1,361張差1張屬正常捨入。⭐三大法人依分項加總合計淨買超7,878張(官方合計欄+7,879,185股)，為 9/07（當時 16,488 張）以來單日最大淨買超——⚠️ 本報須就此設限：已核算 2026-07-01 至 09-18 共 57 個交易日，7,878 張在該區間排名第 5，更大者尚有 7/31 的 23,567 張、9/07 的 16,488 張、7/01 的 11,755 張、8/05 的 9,948 張，故本報僅宣稱「9/07 以來最大」，不宣稱為追蹤期間最大；全市場三大法人合計淨買超NT$1,194.51億。
+(5)⭐⭐技術面連續第2個交易日全面修復，且其中一項已逼近訊號轉折：(a)⭐⭐MACD柱自-8.90大幅收斂至-1.58，收斂幅度7.32大於前一日的4.10、為連2日收斂；DIF自5.32升至8.79、DEA自9.78降至9.58，兩者差距自-4.46收斂至-0.79——即DIF距向上穿越DEA(黃金交叉、負柱轉正)僅差0.79，本報列為次日第一順位檢核。⚠️本欄仍為負值，本報不因「即將轉正」而提前宣告轉強。(b)KDJ的J自+10.53再升36.39點至+46.92，兩個交易日累計自9/16的-17.25回升64.17點；K自24.65升至38.23、D自31.72升至33.89，⭐K已重新高於D(正乖離+4.34)，中止K低於D的空方型態。(c)RSI 14自52.85升4.43點至57.28，連2日上升並穩居50中軸之上。(d)⭐布林帶寬自4.75%轉為擴張至5.02%，中止先前連續收斂——前報曾把「帶寬續收斂」列為唯一未改善項，本日該項亦已改善；上軌2,477／中軌2,417／下軌2,356。⭐口徑驗證：以同一套算法回算9/17已發布值(RSI 52.85／MACD柱-8.90／DIF 5.32／DEA 9.78／K 24.65／D 31.72／J 10.53／MA5 2,396／MA10 2,424／MA20 2,414／MA60 2,396／MA120 2,296／布林2,357-2,414-2,472／5日均量19,381)全數逐項完全複現，確認口徑未漂移後才計算本日。序列為TWSE官方2026-01-02至2026-09-18共173個交易日、不還原除息；KDJ之RSV採STOCK_DAY最高／最低價序列(非收盤價)，布林採母體標準差(ddof=0)。
+(6)⭐均線全面上移且本次無滾動窗口造成的反直覺現象(前報曾出現「股價大漲而MA5反降」的窗口效應)：MA5自2,396升至2,406(滾出9/11的2,410、滾入2,460，(2,460-2,410)÷5＝+10.0)、MA10自2,424升至2,429、MA20自2,414升至2,417(滾出8/21的2,400，(2,460-2,400)÷20＝+3.0)、MA60自2,396升至2,397、MA120自2,296升至2,301，五條全數上升。⭐收盤2,460同時高於全部五條均線，為連續第2個交易日維持此型態，且與最接近的MA10 2,429已拉開至31元(前一日僅高出1元)，站穩程度明顯提升。⚠️惟收盤距布林上軌2,477僅17元，短線已進入通道上緣壓力區；且本日站上均線的推力含指數審核生效日的被動買盤，型態確立仍待次一交易日在無事件干擾下確認。
+(7)⭐期貨與選擇權：⭐台積電個股期CDF 202610(未換月)日盤收2,469(+36點)、結算價2,468、未平倉24,914口(自9/17的25,045口減131口)，對現貨2,460的基差+9點正價差、較9/17的+8點微幅擴大，屬期現同步上漲下的正常現象。⭐台指期TX 202610日盤收47,418、結算價47,428、未平倉101,893口。⚠️⚠️9/18夜盤(9/18 15:00至9/19約05:00、涵蓋美股9/18全場)台指期202610收47,405、較日盤收盤47,418下跌13點幾近持平——⭐該場夜盤涵蓋了費半+2.78%的美股大漲而台指期未跟進，指向外資對台股的續追意願有限，本報判讀為中性偏弱；⚠️且因間隔整個週末，不作方向性結論。⚠️取數註記：TAIFEX因跨週末將9/18夜盤歸入queryDate=2026-09-21的「盤後」列，若誤查queryDate=2026-09-18取到的會是9/17晚間場次，本報已避開此陷阱。⚠️⚠️TXO本日不可與前一日比較：9/18為當週週結算日、未平倉已結清重建，結算後買權未平倉46,401口、賣權35,415口、雙邊81,816口、P/C未平倉比76.32%(TAIFEX pcRatioDown官方，該檔欄位順序為賣權在前、買權在後，本報已依Unicode碼位確認未讀反)；與9/17的76.50%雖數值接近但分屬結算前後的不同基期，數值接近純屬巧合而非「維持穩定」；雙邊合計未平倉自134,872口降至81,816口(-39.3%)正是結算結清的直接結果。⭐可說的只有絕對水位：買權未平倉多於賣權達31%、結構上偏多。
+(8)⭐評價與匯率：TWSE官方BWIBBU 9/18顯示P/E 28.52x、P/B 9.92x、殖利率0.89%(9/17為28.11x／9.78x／0.91%)，財報基準維持115/2未換季。⭐⭐本日評價上升百分之百來自股價：P/E升幅1.46%、P/B升幅1.43%，與股價漲幅+1.44%一致。市值約NT$63.8兆。ADR端P/E約32.1x、P/B約11.2x(依官方值×ADR換算係數推估、非官方申報值)。⭐⭐新台幣9/18收31.8511(四捨五入採31.85)，較9/17的31.8596小幅升值0.027%——⚠️這中止了自9/11起連續5個交易日的貶值，自9/10的31.4640起算的累計貶幅自1.26%收斂至1.23%。⭐ADR溢價自+13.06%收斂至+12.55%：理論平價＝5×2,460÷31.85＝386.19，對ADR市價$434.67之溢價+12.55%，成因為ADR漲幅+1.03%小於台股+1.44%且新台幣小幅升值兩項同向。⚠️⚠️來源分歧須揭露：Yahoo奇摩股市9/18報導另載當日新台幣在岸收盤為31.808，若改採之則理論平價386.70、ADR溢價+12.40%；本報沿用既有序列以維持與前報可比性，並在此並陳另一讀數與其影響。
+(9)⚠️美股與供應鏈：費半9/18連4紅+2.78%(+322.20點)收11,921.69、四日累計+9.45%，⭐領漲結構轉向設備次族群——科林研發+6.98%、應用材料+6.51%、科磊+4.74%、艾司摩爾+3.08%四檔全數跑贏指數，而輝達僅+1.34%、標普+0.17%、那斯達克+0.39%、VIX降至14.81(-4.08%)。⚠️外電(24/7 Wall St，2026-09-18)明確指出當日並無任何設備商發布可解釋漲幅的消息，判讀為超跌反彈(科林研發彈升前一個月曾跌約13%)，本報標示為未能證實成因。⚠️⚠️長期座標：費半11,921.69距2年高點14,634.72(2026-06-22)仍低18.5%，本輪屬修正格局中的反彈而非新高行情。⚠️⚠️高通9/18重挫-5.82%收$177.72為19檔中唯一重挫、且發生在費半大漲的一天，外電歸因為多重利空疊加(前月漲約12%後的獲利了結、蘋果自研基頻進逼致iPhone插槽份額預期自約20%下修且與蘋果相關產品營收預估12月季環比驟降約50%、核心手機晶片營收年減約20%、升息預期轉鷹)；⭐對台積電而言高通與蘋果同為其客戶、份額在客戶間移轉屬中性，本報不視為台積電的直接利空。⚠️美光收$1,015.80(+3.92%)重返千元之上，⚠️但本報已調閱2年日線確認該價並非歷史新高亦非首度站上$1,000(近2年內收盤高於本日者共17個交易日、2年高點為2026-06-25的$1,213.56)，正確說法是「重返千元」而非「突破千元」。
+(10)⭐⭐次日檢核(次一份日報將逐條回覆)：(a)⚠️⚠️第一順位「乾淨量能」——今日為指數審核事件後第一個交易日，量能將首次在無事件干擾下揭露真實買盤。⚠️本報特別聲明門檻不採用含9/18的5日均量23,333張(該均量已被單一極端值灌水，機械套用會得出失真結論)，改用剔除9/18後的四日均量18,943張(9/14 21,521、9/15 15,216、9/16 20,919、9/17 18,117)為乾淨基準：若今日量能站上18,943張且收盤守穩2,435之上，本報將追認9/17-9/18的反彈有買盤支撐；若回落至18,943張之下，則9/18爆量應判定為一次性指數調節。(b)⭐第二順位「MACD能否完成黃金交叉」——DIF 8.79、DEA 9.58、差距-0.79，若今日收盤後DIF高於DEA則MACD柱為9/14轉負以來首度翻正。(c)⭐第三順位「相對強弱能否回復」——9/18落後加權指數0.49個百分點，觀察能否重新領先大盤。(d)⭐第四順位「外資能否連三日買超」。⚠️今日盤中參考(台北時間約09:20、非收盤價，次一份日報將以正式收盤價回頭補正)：2330報2,455、略低於9/18收盤2,460，與夜盤中性偏弱的指示方向一致。</t>
+        </is>
+      </c>
+      <c r="G130" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:G2"/>

</xml_diff>

<commit_message>
daily: 2026-09-22 日報 HTML & Excel 更新
涵蓋 2026-09-21(Mon) 收盤：台股 2330 收 2,480 (+20.00/+0.81%)、量 16,087 張；
ADR TSM 收 445.14 (+2.41%)。

主要判斷：前報兩項第一/二順位檢核一過一不過——MACD 黃金交叉明確完成
(柱 -1.58 → +5.48、DIF 13.00 反超 DEA 10.26，為 9/14 轉負連 5 日以來首度翻正)，
但「乾淨量能」未過門檻 18,943 張 (實際 16,087、差 15.1%)。依前報自訂判準確認
9/18 爆量為一次性指數調節：台積電量能 -60.7% 而全市場僅 -13.1% (4.6 倍)、
成交筆數僅 -0.2% 而股數 -60.7% (大單特徵反向消失)。立場維持中性偏多不上調。

自查與驗收修正六項：
- TAIFEX 漲跌欄基準為「前一場結算價」非收盤價，全文統一改採對收盤價口徑並
  標註官方值 (CDF 日盤 +28 vs +27、夜盤 +25/+1.00% vs +24/+0.96%、
  TX 夜盤 +728/+1.51% vs +704/+1.46%)
- 理論平價 12,400÷31.81=389.8145 應顯示 389.81 (原誤植 389.82)，並說明
  溢價 +14.19% 係以未二次捨入之平價計算
- 交易日計數 7/02–9/18 為 56 日 (原誤寫 55)
- 9 月量能敘述改為可查證值：中位數 20,919 張、區間 14,102–40,893
- 排名類宣稱更正：蘋果非 18 檔漲幅最小 (SK 海力士 +0.59% 才是)、輝達非
  距 2 年高點最近者 (超微與聯發科當日已創 2 年收盤新高)
- 「單月歷史新高」補標為台積電官方新聞稿措辭、非本報自行核算範圍

另補上逐日數值使「連 N 日」宣稱可由報告自身複核 (自營商連 6 日、費半與
輝達、超微連 5 日)。

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -912,7 +912,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-09-21</t>
+          <t>報告更新日期：2026-09-22</t>
         </is>
       </c>
     </row>
@@ -3377,7 +3377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G130"/>
+  <dimension ref="A1:G131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3399,7 +3399,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-09-21</t>
+          <t>最後更新：2026-09-22</t>
         </is>
       </c>
     </row>
@@ -8256,6 +8256,55 @@
         </is>
       </c>
     </row>
+    <row r="131">
+      <c r="A131" s="50" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B131" s="50" t="inlineStr">
+        <is>
+          <t>NT$2,480（9/21收，7/01以來最高）</t>
+        </is>
+      </c>
+      <c r="C131" s="51" t="inlineStr">
+        <is>
+          <t>+0.81%（9/21收，+20.00，落後大盤+1.14%）</t>
+        </is>
+      </c>
+      <c r="D131" s="50" t="inlineStr">
+        <is>
+          <t>US$445.14（9/21收，+2.41%）</t>
+        </is>
+      </c>
+      <c r="E131" s="50" t="inlineStr">
+        <is>
+          <t>16,087（9/21收，-60.7%，未過乾淨門檻18,943）</t>
+        </is>
+      </c>
+      <c r="F131" s="52" t="inlineStr">
+        <is>
+          <t>報告日2026-09-22(Tue)，台股資料為2026-09-21(Mon)官方收盤；ADR、費半與全部美股個股、韓股為9/21正式收盤；期貨為TAIFEX 9/21日盤，另含今晨夜盤(9/21 15:00至9/22約05:00、涵蓋美股9/21全場)。
+(0)⭐兩項閱讀前提：(a)與前一行不同，今晨夜盤為正常平日場次、與今日開盤之間無週末阻隔，指示性已回復平日水準。(b)新台幣匯率採Yahoo TWD=X序列經台北時區換算後之當日值31.8091(本行四捨五入採31.81)，與前一行同一口徑故可比。
+(1)⚠️⚠️本日最重要的事是「MACD金叉達標、但量能檢核未過」這組方向相反的訊號，且本行選擇不因單一指標轉正而上調立場：台股2330官方收NT$2,480(開2,445＝全日最低／高2,485／收2,480，量16,087張、額NT$397.73億、69,432筆，TWSE STOCK_DAY確認)，漲跌價差+20.00(對9/18收盤2,460、+0.81%)。⭐2,480為2026-07-01(收2,505)以來最高收盤，本行已核算7/02至9/18共56個交易日無一收盤達2,480。⚠️⚠️但成交量16,087張低於前一份日報明訂的乾淨門檻18,943張達15.1%，依前報自訂且已白紙黑字寫下的判準「若量能回落至18,943張之下，則9/18的爆量應被判定為一次性的指數調節，反彈的量能基礎不成立」，本行今日據此執行該判定。
+(2)⭐⭐9/18爆量確認為一次性指數調節，且本日的證據為雙向驗證而非單一數字：(a)台積電自身量能自40,893張暴跌至16,087張(-60.7%)，而同日全市場成交股數僅自12,052,158,761股降至10,478,763,517股(-13.1%，TWSE FMTQIK官方)，回落幅度為全市場的4.6倍；(b)成交筆數自69,571筆降至69,432筆(-0.2%)幾乎持平而股數減60.7%，即9/18判定為「大單特徵」的依據(筆數僅增13.0%而股數增125.7%)於本日完全反向複現。⚠️減輕因素須並陳：16,087張在2026年174個交易日中為第8低，但2026年全年成交量中位數為35,660張、9月15個交易日的成交量中位數為20,919張(區間14,102~40,893張)、較全年中位數低約41%，近期量能整體已處年度低檔區，不宜全部解讀為本日特有的買盤退場。
+(3)⭐⭐逐條履行前一份日報所訂五項檢核，結果為三項通過、一項未通過、一項部分通過：(a)⚠️⚠️第一順位「乾淨量能」——部分通過。門檻為量能站上18,943張且收盤守穩2,435，實際為量能16,087張(未過、差15.1%)、收盤2,480(大幅守穩、高出45元)。(b)⭐⭐第二順位「MACD黃金交叉」——通過：DIF自8.79升至13.00、DEA自9.58升至10.26，DIF反超DEA達2.74，柱體自-1.58翻正為+5.48，為9/14轉負後(9/14 -4.77、9/15 -9.61、9/16 -13.00、9/17 -8.90、9/18 -1.58)連續5個交易日負值以來的首度翻正。(c)⚠️第三順位「相對強弱能否回復」——未回復：台積電+0.81%仍落後加權指數+1.14%(TWSE FMTQIK官方47,180.75→47,718.84、+538.09點)，連2日落後，惟落後幅度自0.49個百分點收斂至0.33個百分點。(d)⭐第四順位「外資能否連三日買超」——通過：外資買超2,689張，連3日合計13,522張。(e)⭐夜盤指示——兌現：前報判9/18夜盤中性偏弱，9/21果然開低至2,445；⚠️惟前報所引盤中參考價2,455(台北09:20)低於最終收盤2,480達25元，本行依約補正，並記錄教訓：開盤後20分鐘的盤中價對全日方向指示力有限。
+(4)⭐⭐籌碼面連3日淨買超但金額規模縮小：(a)外資對台積電買超2,689張(TWSE T86官方買進9,832,887股／賣出7,143,383股／淨+2,689,504股，依既定口徑向零截斷)，以2,480元計約NT$66.70億，僅為9/18的NT$148.57億的44.9%。(b)⭐惟集中度回升：TWSE BFI82U顯示9/21全市場外資淨買超NT$204.79億，台積電單檔占32.6%，與9/18的17.1%相比明顯回升，與「指數審核事件結束後外資配置重新向台積電集中」的判讀一致。(c)投信買超734張(連2日：9/18 +478、9/21 +734)、自營商買超614張(連6日：9/14 +196、9/15 +350、9/16 +762、9/17 +509、9/18 +1,361、9/21 +614)；自營商分項自行買賣+438,552股(+438張)、避險+176,050股(+176張)，向零截斷後相加614張，與官方合計欄換算值一致、本日無1張差異。(d)⭐三大法人依分項加總合計淨買超4,037張(官方合計欄+4,038,712股)，為連3日淨買超、三日合計17,159張；全市場三大法人合計淨買超NT$478.05億。⚠️本行未核算4,037張在追蹤期間的排名，不作任何「最大」類宣稱。
+(5)⭐⭐技術面完成本波最關鍵的訊號轉折，四項指標全數改善：(a)⭐⭐⭐MACD黃金交叉完成，見(3)(b)。(b)RSI 14自57.28升2.33點至59.61，連3日上升；⭐升幅逐日遞減(6.66→4.43→2.33)，本行讀為推力遞減而非加速轉強，59.61距70超買區仍有10.39點。(c)KDJ續強：K自38.23升至55.92、D自33.89升至41.23，K對D正乖離自+4.34擴大至+14.69；J自46.92升至85.30。⚠️本行就J值設限：已核算2026年174個交易日中J&gt;85者達43日(約四分之一)，以本標的自身分布而言並非罕見極端，不宜單獨據此判定過熱。(d)布林帶寬自5.02%續擴張至5.23%(連2日擴張)，上軌2,485／中軌2,422／下軌2,359。⚠️⚠️收盤2,480距上軌僅5元(0.2%)，短線緩衝空間已極度壓縮。⭐口徑驗證：以同一套算法回算9/18已發布值(RSI 57.28／MACD柱-1.58／DIF 8.79／DEA 9.58／K 38.23／D 33.89／J 46.92／MA5 2,406／MA10 2,429／MA20 2,417／MA60 2,397／MA120 2,301／布林2,356-2,417-2,477／5日均量23,333)全數逐項完全複現，確認口徑未漂移後才計算本日。序列為TWSE官方2026-01-02至2026-09-21共174個交易日、不還原除息；KDJ之RSV採STOCK_DAY最高／最低價序列(非收盤價)，布林採母體標準差(ddof=0)。
+(6)⭐均線全面上移且無滾動窗口造成的反直覺現象：MA5自2,406升至2,426(滾出9/14的2,380、滾入2,480，(2,480-2,380)÷5＝+20.0)、MA10自2,429升至2,431、MA20自2,417升至2,422(滾出8/24的2,375，(2,480-2,375)÷20＝+5.25)、MA60自2,397升至2,399、MA120自2,301升至2,307，五條全數上升。⭐收盤2,480連續第3個交易日同時高於全部五條均線，且與最接近的MA10 2,431拉開至49元(9/18為31元、9/17僅1元)。⚠️惟MA10(2,431)仍高於MA5(2,426)，完整多頭排列尚未成形。
+(7)⭐期貨與選擇權：(a)台積電個股期CDF 202610日盤收2,496(較9/18日盤收盤2,469漲27點；TAIFEX官方漲跌價欄為+28、係對前一日結算價2,468計算，+1.13%)、結算價2,495、未平倉24,793口(自9/18的24,914口減121口)，對現貨2,480的基差+16點正價差、較9/18的+9點擴大7點，期貨漲幅大於現貨為基差擴大的直接成因。(b)外資臺股期貨多空未平倉淨額-74,081口(多10,318／空84,399，TAIFEX官方)，較9/18的-76,110口減少2,029口淨空單，連2日收斂(⚠️核算範圍僅及9/16起)。(c)⚠️台指選擇權可比性須設限：9/18為週結算日、其81,816口為結算後初始重建值，9/21為重建後第一個完整交易日，雙邊合計增至120,569口(+47.4%)主要反映建倉累積。⭐可讀的是結構：賣權未平倉自35,415口增至59,117口(+66.9%)、買權自46,401口增至61,452口(+32.4%)，賣權增幅為買權的2.1倍，P/C比自76.32%升至96.20%，買權多於賣權的優勢自31%收斂至4%。⚠️本週下一次週結算為9/23(週三)。(d)⭐⭐今晨夜盤方向明確偏多：個股期CDF 202610收2,520(較日盤收盤2,496漲24點、+0.96%)、台指期TX 202610收48,781(較日盤收盤48,077漲704點、+1.46%)；⚠️TAIFEX官方漲跌欄記為+25/+1.00%與+728/+1.51%，係對日盤結算價2,495與48,053計算，本行一律採對日盤收盤價口徑。⚠️取數註記：TAIFEX以夜盤結束日標記場次，須查queryDate=2026-09-22的「盤後」列。
+(8)⭐評價與匯率：TWSE官方BWIBBU 9/21顯示P/E 28.75x、P/B 10.00x、殖利率0.89%(9/18為28.52x／9.92x／0.89%)，財報基準維持115/2未換季。⭐本日評價上升百分之百來自股價：P/E與P/B升幅均為0.81%，與股價漲幅+0.81%完全一致。市值約NT$64.3兆。⚠️本行就P/B設限：並未核算「10.00x是否為歷史或區間高點」，不作任何創高宣稱，僅陳述該值本日恰為整數10.00x。⭐新台幣31.8091(採31.81)較9/18的31.8511升值0.13%，連2日升值，自9/10的31.4640起算累計貶幅自1.23%收斂至1.10%。⚠️ADR溢價自+12.55%擴大至+14.19%(理論平價＝5×2,480÷31.81＝389.8145(顯示值389.81)，對市價$445.14)，中止連2日收斂。⚠️⚠️期間報酬表有兩處基準漂移造成的假跳動：台積電1個月報酬自+3.36%降至+2.90%係基準日自8/18(2,380)移至8/21(2,410)所致，加權指數1個月自+4.13%跳升至+5.52%亦主要來自基準自45,308.68降至45,224.29，兩者差距擴大(自-0.77個百分點至-2.62個百分點)有相當部分為機械效果。
+(9)⭐⭐美股與供應鏈為本行追蹤以來最一面倒的一天，19檔中18漲1跌：費半9/21連5紅+4.29%(+511.48點)收12,433.17、五日累計+11.70%，而標普僅+1.49%、那斯達克+2.26%，VIX 14.87(+0.41%)。⭐催化事件兩說並陳：(a)Bloomberg／Investing.com歸因於Meta新AI代理人Muse上線後採用率超預期(9/19單日美國下載26.4萬次、連3日逾20萬次)，引爆「AI需求帶動伺服器CPU需求」樂觀情緒；(b)FinancialContent／StockStory歸因於美中貿易緊張緩解、油價下跌與公債殖利率走低，未提及Meta。兩說可能同時成立，本行並陳不作取捨。⭐⭐漲幅前四名全為美股處理器陣營(CPU、IP授權與手機晶片)：Arm +17.16%($322.90)、英特爾+12.14%($121.78)、超微+9.95%($615.52)、高通+9.29%($194.23)。⚠️連續三個交易日領漲族群三度輪換(9/17 AI晶片設計→9/18設備→9/21 CPU／IP)，本行判讀為情緒驅動、缺乏單一主線。⭐超微$615.52經本行以近2年499個交易日核算確認為近2年收盤新高(前高2026-06-30的$580.91)；外電另稱創歷史新高並首度站上1兆美元市值，該兩項標示為引述外電、非本行證實。⭐聯發科收5,010元(+6.37%)經本行以近2年486個交易日核算同為近2年收盤新高。⚠️唯一下跌者為華邦電-3.06%(收174.00)，而該檔正是9/18漲幅第二大者(+5.59%)，回吐逾半。⭐TSM ADR收$445.14(+2.41%)為7/06以來最高收盤，⚠️惟連2日落後費半(本日落後1.88個百分點)。
+(10)⭐⭐次日檢核(次一份日報將逐條回覆)：(a)⚠️⚠️第一順位仍為量能，門檻重設——改用剔除9/18極端值後、含9/21的四日均量17,585張(9/15 15,216、9/16 20,919、9/17 18,117、9/21 16,087)。若今日量能站上17,585張且收盤守穩2,445之上，本行將視為量能開始補上、價漲量縮的背離解除；若續低於17,585張，則不論股價漲跌一律維持「量能基礎不成立」的判定、立場不上調。(b)⚠️⚠️第二順位為布林上軌2,485(收盤距上軌僅5元)：若收盤站上並守住2,485，記錄為通道外緣突破，並同時觀察J值(85.30)是否越過90；若在2,485之下遇壓回落，則9/21的新高視為單日衝高而非有效突破。(c)⭐第三順位為相對強弱能否由落後轉為領先；若連3日落後，資金輪動至非台積電標的的型態將獲確認。(d)⭐第四順位為外資能否連四日買超，且關注金額而非次數(買超金額已自NT$148.57億腰斬至NT$66.70億)。(e)⚠️9/23(週三)為台指選擇權週結算日，次一份日報引用P/C比與未平倉時須留意重置效應。
+(11)⭐本行立場維持「中性偏多」不再上調，理由單一且明確：量能檢核未過，價漲量縮的背離尚未解除，且收盤距布林上軌僅5元、短線已無緩衝空間。</t>
+        </is>
+      </c>
+      <c r="G131" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:G2"/>

</xml_diff>

<commit_message>
daily: 2026-09-23 日報 HTML & Excel 更新
涵蓋 2026-09-22(Tue) 收盤：台股 2330 收 2,460 (-20.00/-0.81%)、量 22,010 張；
ADR TSM 收 452.00 (+1.54%)。

主要判斷：開高 2,505、盤中 2,510 (6/23 以來最高盤中價) 後收在全日最低；
前報檢核中布林上軌、相對強弱 (連 3 日落後、0.98pp)、外資連四買三項未過，
量能字面過但量增出現在黑 K。外資賣超 4,329 張而全市場外資淨買超 453.21 億。
MA5 穿越 MA10、五線恢復完整多頭排列。立場自中性偏多下修為中性。
另記 9/25、9/28 休市與 9/23 週結算。

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -912,7 +912,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-09-22</t>
+          <t>報告更新日期：2026-09-23</t>
         </is>
       </c>
     </row>
@@ -3377,7 +3377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G131"/>
+  <dimension ref="A1:G132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3399,7 +3399,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-09-22</t>
+          <t>最後更新：2026-09-23</t>
         </is>
       </c>
     </row>
@@ -8305,6 +8305,48 @@
         </is>
       </c>
     </row>
+    <row r="132">
+      <c r="A132" s="53" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B132" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,460（9/22收，收在全日最低；盤中高2,510為6/23以來最高）</t>
+        </is>
+      </c>
+      <c r="C132" s="56" t="inlineStr">
+        <is>
+          <t>-0.81%（9/22收，-20.00，落後大盤+0.17%）</t>
+        </is>
+      </c>
+      <c r="D132" s="53" t="inlineStr">
+        <is>
+          <t>US$452.00（9/22收，+1.54%，6/30以來最高收盤）</t>
+        </is>
+      </c>
+      <c r="E132" s="53" t="inlineStr">
+        <is>
+          <t>22,010（9/22收，+36.8%，量增但收黑K）</t>
+        </is>
+      </c>
+      <c r="F132" s="55" t="inlineStr">
+        <is>
+          <t>報告日2026-09-23(Wed)，台股資料為2026-09-22(Tue)官方收盤；ADR、費半與美股個股、韓股為9/22正式收盤；期貨為TAIFEX 9/22日盤，另含今晨夜盤(9/22 15:00至9/23約05:00)。
+(1)⚠️⚠️開高走低收最低：台股2330開2,505(跳空+25)、盤中高2,510(6/23以來最高盤中價)、收2,460＝全日最低(-20、-0.81%)，開收跌幅45元為7/29以來最大；⚠️惟「跳空開高、收最低」在2026年已出現18次，非罕見型態。媒體歸因於9/25中秋、9/28教師節連假前獲利了結(本報無法證實動機)。
+(2)⭐⭐前報六項檢核：量能字面通過(22,010張&gt;17,585、收盤守2,445)但量增出現在黑K、實質存疑；布林上軌未通過(盤中越2,490上軌、收盤退回)；相對強弱未通過且觸發確認(連3日落後加權+0.17%，落後0.98pp)；外資連四買未通過(轉賣4,329張約NT$106.51億，而全市場外資淨買超NT$453.21億)；夜盤只兌現開盤方向。
+(3)⭐技術：MA5 2,441穿越MA10 2,430(8/26以來首度)、五線恢復完整多頭排列(9/14以來首度)、收盤連4日站上全部均線；MACD柱+6.87續擴大(屬EMA慣性)、RSI 56.30中止連3升、J 80.98回落。
+(4)⭐籌碼與衍生品：投信-405張、自營+467張(連7日)、三大法人-4,267張中止連3買；個股期CDF日盤2,489、基差+29；外資台指期淨空擴大至-75,568口；今晨夜盤CDF收2,515(+26)。ADR溢價擴大至+16.64%，新台幣31.7384連3日升值。
+(5)立場自「中性偏多」下修為「中性」。次日檢核：收盤能否守2,445(跌破則升級為短線反轉)、外資賣超是否擴大；9/23週結算、9/24連假前最後交易日、美光美東9/30財報。</t>
+        </is>
+      </c>
+      <c r="G132" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:G2"/>

</xml_diff>

<commit_message>
daily: 2026-09-24 日報 HTML & Excel 更新
涵蓋 2026-09-23(Wed) 收盤：台股 2330 收 2,500 (+40.00/+1.63%)、量 22,818 張；
ADR TSM 收 446.57 (-1.20%)。

主要判斷：開盤即最低 2,475、收 2,500 為 7/01 以來最高收盤；前報三項主要檢核
(守 2,445 且站回 2,480、外資轉買 7,123 張、領先加權 0.88pp) 全數朝正面兌現，
9/22 黑 K 改判為連假前單日部位調整。惟台股收盤後美國 10 年期殖利率升至 5.11%、
費半 -1.23%，今晨夜盤 CDF 2,492 (-18)；J 值 100.11、量低於均量。立場維持中性。
另更正 pe_nyse/pb_nyse 恢復既定公式 (9/21、9/22 兩日未依公式)。
已經 fresh-context 驗收 (官方 TWSE/TAIFEX/Yahoo 重算)，J>=100 日數敘述依驗收意見修正。

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -912,7 +912,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-09-23</t>
+          <t>報告更新日期：2026-09-24</t>
         </is>
       </c>
     </row>
@@ -3377,7 +3377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G132"/>
+  <dimension ref="A1:G133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3399,7 +3399,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-09-23</t>
+          <t>最後更新：2026-09-24</t>
         </is>
       </c>
     </row>
@@ -8347,6 +8347,48 @@
         </is>
       </c>
     </row>
+    <row r="133">
+      <c r="A133" s="50" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B133" s="50" t="inlineStr">
+        <is>
+          <t>NT$2,500（9/23收，7/01以來最高收盤；開盤＝全日最低2,475）</t>
+        </is>
+      </c>
+      <c r="C133" s="51" t="inlineStr">
+        <is>
+          <t>+1.63%（9/23收，+40.00，領先大盤+0.75%）</t>
+        </is>
+      </c>
+      <c r="D133" s="50" t="inlineStr">
+        <is>
+          <t>US$446.57（9/23收，-1.20%，中止連5漲；美債10年期殖利率升至5.11%）</t>
+        </is>
+      </c>
+      <c r="E133" s="50" t="inlineStr">
+        <is>
+          <t>22,818（9/23收，+3.7%，低於5日均量4.9%）</t>
+        </is>
+      </c>
+      <c r="F133" s="52" t="inlineStr">
+        <is>
+          <t>報告日2026-09-24(Thu)，台股資料為2026-09-23(Wed)官方收盤；ADR、費半與美股個股、韓股為9/23正式收盤；期貨為TAIFEX 9/23日盤，另含今晨夜盤(9/23 15:00至9/24約05:00)。
+(1)⭐⭐收復：台股2330開盤即全日最低2,475、收2,500(+40、+1.63%)，為7/01以來最高收盤(2026年收盤≥2,500僅6/22、7/01與本日)；外資轉買7,123張(約NT$178.1億，占全市場外資淨買超NT$373.13億約47.7%)，領先加權+0.75%達0.88pp。
+(2)⭐⭐前報六項檢核：價格分界2,445守住且收盤站回2,480之上→9/22黑K改判為連假前單日部位調整；外資轉買→9/22賣超視為單日調節；相對強弱中止連3日落後→輪動判定降級為觀察中；夜盤開盤與收盤方向皆兌現；9/23週結算P/C 79.83%只讀水位。
+(3)⭐技術：MACD柱+12.28(9/09以來最大)、RSI 60.97(7/01以來最高)、⚠️J 100.11(8/13以來首度站上100)；五線完整多頭排列連2日、收盤距布林上軌2,501僅1.38元；量22,818張低於5日均量，屬價漲量平。
+(4)⚠️⚠️台股收盤後美國10年期公債殖利率升至5.11%(CNN稱19年來首見)，費半-1.23%中止連6紅、ADR-1.20%收$446.57，溢價收斂至+13.18%；今晨夜盤CDF收2,492(-18)、台指期-427點；外資台指期淨空擴大至-76,084口。
+(5)立場維持「中性」。次日檢核：收盤能否守2,475(守住則回升中性偏多、跌破2,460則9/23漲幅全數回吐)；9/24為連假前最後交易日，9/25、9/28休市、美股照常交易三日；美光美東9/30財報。</t>
+        </is>
+      </c>
+      <c r="G133" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:G2"/>

</xml_diff>

<commit_message>
daily: 2026-09-29 日報 HTML & Excel 更新
連假後首個交易日：台股數據 9/24（9/25 中秋、9/28 教師節休市，9/25 排程未執行、本份一併補記）；美股 9/24–9/28 三日、TAIFEX 9/24 日盤與 9/29 今晨夜盤。

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="600" firstSheet="0" activeTab="6" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="封面總覽" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="財務摘要" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="營收結構分析" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026展望" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="股息記錄" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="風險評估" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="每日更新記錄" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="封面總覽" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="財務摘要" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="營收結構分析" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="2026展望" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="股息記錄" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="風險評估" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="每日更新記錄" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -912,7 +912,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-09-24</t>
+          <t>報告更新日期：2026-09-29</t>
         </is>
       </c>
     </row>
@@ -3377,7 +3377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G133"/>
+  <dimension ref="A1:G134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3399,7 +3399,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-09-24</t>
+          <t>最後更新：2026-09-29</t>
         </is>
       </c>
     </row>
@@ -8389,6 +8389,49 @@
         </is>
       </c>
     </row>
+    <row r="134">
+      <c r="A134" s="53" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B134" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,475（9/24收，連假前最後交易日；低開2,480、收盤恰落在分界2,475）</t>
+        </is>
+      </c>
+      <c r="C134" s="56" t="inlineStr">
+        <is>
+          <t>-1.00%（9/24收，-25.00，落後大盤-0.28%）</t>
+        </is>
+      </c>
+      <c r="D134" s="53" t="inlineStr">
+        <is>
+          <t>US$452.88（9/28收，+0.50%；連假三日累計+1.41%；美債10年期殖利率升至5.24%）</t>
+        </is>
+      </c>
+      <c r="E134" s="53" t="inlineStr">
+        <is>
+          <t>14,558（9/24收，-36.2%，2026年第6低、低於5日均量37.4%）</t>
+        </is>
+      </c>
+      <c r="F134" s="55" t="inlineStr">
+        <is>
+          <t>報告日2026-09-29(Tue)，連假後首個交易日。台股資料為2026-09-24(Thu)官方收盤(9/25中秋、9/28教師節休市；⚠️9/25排程未執行、本則一併補記9/24行情)；ADR、費半與美股個股為9/28正式收盤(另記連假期間美股9/24、9/25、9/28三日)；韓股為9/28收盤(9/24-25休市)；期貨為TAIFEX 9/24日盤，另含今晨夜盤(9/28 15:00至9/29約05:00)，期交所9/24晚間至9/28全無交易。
+(1)⚠️9/24台股2330低開2,480、收2,475(-25、-1.00%)，恰落在前報第一順位分界2,475上；量14,558張為2026年第6低(-36.2%)，外資轉賣4,667張(約NT$115.5億，占全市場外資淨賣超NT$329.65億約35.0%)，投信連3賣1,287張、自營連9買242張，三大法人淨賣5,712張；落後加權-0.28%達0.72pp，聯發科+1.93%(連4日近2年新高)、日月光+0.87%逆勢。
+(2)⭐⭐前報六項檢核：分界2,475字面守住但量縮無效檢驗→本報首次在字面達標時不依判準上調、維持「中性」並說明理由；外資轉賣且全市場同向→總經面普遍撤出；相對強弱未通過；夜盤開盤與收盤方向皆兌現(4日實證開盤4/4、收盤2/4)；技術過熱如期提醒；連假提醒適用。
+(3)⭐技術：MACD柱+11.61翻正以來首度縮小(DIF 19.92續升)、RSI 56.88、J自100.11退回93.37；收盤恰等於MA5 2,475，五線多頭排列連3日但站在臨界點；布林2,358-2,433-2,507、寬度6.10%。
+(4)⚠️⚠️連假期間美股三日：10年期殖利率5.162%→5.184%(9/25盤中5.230%為2007年以來最高)→5.240%；費半-0.33%/+1.41%/-1.61%三日累計-0.55%；9/28 AI安全疑慮(OpenAI代理式模型逃出容器)使Arm-8.70%、高通-7.17%、英特爾-5.67%、超微-3.61%、美光-2.61%，輝達+1.68%(加碼1,500億美元庫藏股)、ADR+0.50%收$452.88、艾司摩爾+1.58%逆勢；韓股9/28三星-5.43%、SK海力士-5.05%。ADR溢價擴至+16.30%(時差效果)。今晨夜盤CDF收2,505(+9)、台指期-167點；外資台指期淨空連3日擴大至-77,031口。
+(5)⭐消息：經濟日報9/28報導大廠追加2奈米訂單10-20%、年底月產能上看12萬片；Digitimes 9/24證實高通旗艦晶片採台積電2奈米；台積電赴美投資第7度核准累計440億美元；Q3法說會官方確認10/15(四)14:00-15:30、緘默期10/5-10/14。
+(6)立場維持「中性」。次日檢核：收盤守2,475且量能&gt;9月中位數21,025張則回升中性偏多；跌破2,460則五線紀錄中斷、下調展望；外資是否回補；台積電能否領先大盤(夜盤指示個股偏多、大盤偏空)；美光美東9/30財報、週選9/30結算、9月營收約10/10。</t>
+        </is>
+      </c>
+      <c r="G134" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:G2"/>

</xml_diff>

<commit_message>
daily: 2026-09-30 日報 HTML & Excel 更新
台股 9/29 連假後首日平盤 2,475（量 26,893 張）、外資續賣 3,736 張；立場依前報判準上調為中性偏多。
全數以 TWSE/TAIFEX/Yahoo 官方 API 取數；60 日 beta 改採回歸法（0.99），新聞中 2 則與官方收盤矛盾者剔除。

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -912,7 +912,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-09-29</t>
+          <t>報告更新日期：2026-09-30</t>
         </is>
       </c>
     </row>
@@ -3377,7 +3377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G134"/>
+  <dimension ref="A1:G135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3399,7 +3399,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-09-29</t>
+          <t>最後更新：2026-09-30</t>
         </is>
       </c>
     </row>
@@ -8432,6 +8432,49 @@
         </is>
       </c>
     </row>
+    <row r="135">
+      <c r="A135" s="50" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B135" s="50" t="inlineStr">
+        <is>
+          <t>NT$2,475（9/29收，連假後首日平盤；開＝低＝收2,475、高2,495 T字線）</t>
+        </is>
+      </c>
+      <c r="C135" s="61" t="inlineStr">
+        <is>
+          <t>0.00%（9/29收，0.00，領先大盤+0.82pp；加權-0.82%）</t>
+        </is>
+      </c>
+      <c r="D135" s="50" t="inlineStr">
+        <is>
+          <t>US$456.94（9/29收，+0.90%；費半+1.32%；ADR溢價+17.72%）</t>
+        </is>
+      </c>
+      <c r="E135" s="50" t="inlineStr">
+        <is>
+          <t>26,893（9/29收，+84.7%，高於9月中位數21,025張、5日均量1.31倍）</t>
+        </is>
+      </c>
+      <c r="F135" s="52" t="inlineStr">
+        <is>
+          <t>報告日2026-09-30(Wed)。台股資料為2026-09-29(Tue，連假後首個交易日)TWSE官方收盤；ADR、費半與美股個股為9/29正式收盤；韓股為9/29收盤；期貨為TAIFEX 9/29日盤，另含今晨夜盤(9/29 15:00至9/30約05:00)。今日9/30為週選結算日、美光美東9/30盤後財報。
+(1)⭐9/29台股2330開＝低＝收2,475(高2,495、0.00%)，量26,893張(+84.7%、成交金額NT$666.59億、62,248筆)，加權-392.64點(-0.82%)收47,631.96、聯發科-7.10%、日月光-1.72%，台積電領先大盤0.82pp。外資續賣3,736張(連2日合計8,403張、約NT$92.6億；全市場外資賣超NT$632.01億【媒體數】、台積電占約14.7%)、投信結束連3賣轉買628張、自營連10買117張，三大法人合計-2,991張。P/E 28.69x、P/B 9.98x、殖利率0.89%不變。
+(2)⭐⭐前報七項檢核：「守2,475且量能&gt;21,025張→回升中性偏多」通過，本報依判準上調為「中性偏多」；「收盤≥2,475延續五線紀錄」字面通過但MA5已上移至2,478、收盤低於MA5三元，紀錄止於6日；跌破2,460未觸發；外資未回補；台積電領先大盤兌現；美光財報、週選結算如期提醒。回撤條件：收盤跌破MA10 2,442或外資第3日賣超逾5,000張即退回中性。
+(3)⭐技術：RSI 56.88不變(平盤數學結果)、MACD柱+10.33連2日縮小(DIF 20.56續升)、K 72.13/D 64.09/J 88.23；MA5 2,478/MA10 2,442/MA20 2,435/MA60 2,402/MA120 2,329五線多頭排列連4日；布林2,359-2,435-2,511、寬6.26%；5日均量20,473張。
+(4)⭐美股9/29費半+1.32%收12,629.16(回補9/28跌幅八成)，設備四檔全數大漲(應材+5.19%、科磊+3.89%、艾司摩爾+3.56%、科林+2.99%，皆創1個月新高)，Arm+3.65%、美光+1.05%、博通+1.58%；蘋果-2.66%、高通-1.80%、輝達-0.72%偏弱；ADR+0.90%收$456.94。韓股9/29三星+0.93%、SK海力士-0.17%。新台幣9/29收31.876(貶9.6分)。今晨夜盤個股期收2,520(+29、+1.16%)、台指期+698點(+1.46%)同向偏多；外資台指期淨空-79,029口連4日擴大；選擇權PCR 0.75(週結算前收斂)。
+(5)⭐消息：外電傳台積電美國第二園區落腳德州規劃6座廠(未經證實)；美10年期殖利率逼近5.2%、市場定價Fed 10月升息(^TNX官方收盤未取得)；美國CR已延長至12/11、關門風險低；Q3法說會10/15、9月營收約10/10。
+(6)立場上調為「中性偏多」(附保留)。次日檢核：收復2,500並站上MA5→上影線視為洗盤；跌破2,442或外資第3日賣逾5,000張→退回中性；夜盤2,520/+698指示能否兌現；投信轉買、自營連10買能否延續；美光財報(台北10/1凌晨)；週選結算後PCR與外資部位重讀。</t>
+        </is>
+      </c>
+      <c r="G135" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:G2"/>

</xml_diff>

<commit_message>
daily: 2026-10-01 日報 HTML & Excel 更新
資料日 9/30：2330 收 2,480（+0.20%，量 34,282 張）、ADR 456.19（-0.16%）。
全程 TWSE/Yahoo/TAIFEX 官方 API 取數；BFI82U 全市場法人金額改採官方值；
DERIVATIVES 選擇權欄位明示為台指選擇權全市場口徑並另列 CDO 近月數據。

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -912,7 +912,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-09-30</t>
+          <t>報告更新日期：2026-10-01</t>
         </is>
       </c>
     </row>
@@ -3377,7 +3377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G135"/>
+  <dimension ref="A1:G136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3399,7 +3399,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-09-30</t>
+          <t>最後更新：2026-10-01</t>
         </is>
       </c>
     </row>
@@ -8475,6 +8475,49 @@
         </is>
       </c>
     </row>
+    <row r="136">
+      <c r="A136" s="53" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B136" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,480（9/30收，+5；開2,495高2,510收最低2,480，放量黑K）</t>
+        </is>
+      </c>
+      <c r="C136" s="54" t="inlineStr">
+        <is>
+          <t>+0.20%（9/30收，+5.00，落後大盤0.45pp；加權+0.65%）</t>
+        </is>
+      </c>
+      <c r="D136" s="53" t="inlineStr">
+        <is>
+          <t>US$456.19（9/30收，-0.16%；費半-0.00%；ADR溢價+17.17%）</t>
+        </is>
+      </c>
+      <c r="E136" s="53" t="inlineStr">
+        <is>
+          <t>34,282（9/30收，+27.5%，高於9月中位數21,326張、5日均量1.42倍）</t>
+        </is>
+      </c>
+      <c r="F136" s="55" t="inlineStr">
+        <is>
+          <t>報告日2026-10-01(Thu)。台股資料為2026-09-30(Wed，第三季最後交易日)TWSE官方收盤；ADR、費半與美股個股為9/30正式收盤(Yahoo meta 16:00 ET)；韓股為9/30收盤；期貨為TAIFEX 9/30日盤＋今晨夜盤(9/30 15:00至10/1約05:00)；匯率採台北外匯9/30收盤31.852；全市場法人金額採BFI82U官方。
+(1)⚠️9/30台股2330放量34,282張(+27.5%、金額NT$853.89億、83,797筆)開高走低：開2,495、盤中2,510(＝6/22全年最高收盤價位)後收全日最低2,480(+5、+0.20%)，上漲黑K；加權+308.17點(+0.65%)收47,940.13，台積電落後0.45pp；2,495–2,510自9/22起三度上攻未站穩，壓力區依前報判準確立。
+(2)⭐⭐前報六項檢核：收復2,500半通過(盤中收復、收盤未站上，但站回MA5 2,478)；回撤條件(MA10 2,442／外資第3日賣逾5,000張)未觸發；夜盤2,520指示開+20收+5兩端方向兌現(累計開5/6收3/6)；投信+761連2買、自營+399連11買延續；美光FQ4財報大超預期(營收US$542.3億、資料中心年增逾11倍、指引US$615億、盤後約+12%【媒體數】)；週選結算後台指選擇權P/C 80.57%。
+(3)⭐籌碼：外資轉買702張(買25,569,109股／賣24,866,515股，中止連2日賣超8,403張)，三大法人合計+1,864張(9/23以來首度淨買超)；全市場三大法人+NT$403.88億(外資+308.57／投信+82.91／自營+12.40，BFI82U官方)，台積電僅占外資買超5.6%；外資台指期淨空-78,151口(收斂878口、中止連4日擴大)。
+(4)⭐技術(TWSE官方序列179日自算)：RSI 57.54、MACD柱+9.34連3日縮小(DIF 21.23連6升／DEA 16.57)、K 74.02／D 67.40／J 87.25(連3日回落)；MA5 2,478／MA10 2,452／MA20 2,439／MA60 2,403／MA120 2,333五線多頭連5日，收盤站回MA5；布林2,362–2,439–2,516；5日均量24,112張。衍生品：個股期日盤收2,500(+9)、OI 25,063、基差+20，今晨夜盤收2,505(+5)；台指期48,330(+1.15%)、夜盤48,298；CDO近月call 190／put 109口、最大痛點2,500(樣本小)。
+(5)⭐美股9/30費半-0.54點(-0.00%)收12,628.62、ADR -0.16%收$456.19(溢價+17.17%、自17.72%收斂)；19檔供應鏈10漲9跌：科林+1.44%、英特爾+3.71%、蘋果+1.10%、輝達+0.51%；艾司摩爾-1.24%、科磊-0.81%、Amkor-3.25%、Arm-1.37%(五日-12.90%)；台股日月光+2.33%、華邦電+3.16%、聯發科+0.20%；韓股SK海力士+0.62%、三星-1.47%。消息：美10年期殖利率盤中5.29%創2007年來新高【媒體數】、8月PCE年增3.4%降溫但道瓊-0.86%；AMD 82億美元收購World Labs；新台幣9月貶0.59%、外資9月賣超台股429億【媒體數】。BWIBBU P/E 28.75x／P/B 10.00x／殖利率0.89%。
+(6)立場維持「中性偏多」，首要保留改為2,495–2,510壓力區三度受阻與放量黑K(前報頭部警訊字面成立、定為弱化版)。次日檢核：守2,475(破且量增→頭部確認、退回中性)；跌破MA10 2,452或外資單日賣逾5,000張→退回中性；收≥2,510且量≥24,112張→上調；夜盤2,505指示兌現；美光10/1正式收盤核對；外資能否連2買且集中回台積電。9月營收約10/10(官方未公告)、緘默期10/5起、Q3法說10/15。</t>
+        </is>
+      </c>
+      <c r="G136" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:G2"/>

</xml_diff>

<commit_message>
daily: 2026-10-02 日報 HTML & Excel 更新
台股 10/1 收 2,510（+1.21%）平 2026 年最高收盤、量縮 39.7%；外資連 2 買 3,090 張；
ADR 459.20（+0.66%）、費半 +1.59%；美光正式收盤 +3.03%。立場維持中性偏多、不上調。
全程 TWSE/Yahoo/TAIFEX 官方 API 取數，fresh 驗收者 10 項全過。

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="600" firstSheet="0" activeTab="6" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="封面總覽" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="財務摘要" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="營收結構分析" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026展望" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="股息記錄" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="風險評估" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="每日更新記錄" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="封面總覽" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="財務摘要" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="營收結構分析" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="2026展望" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="股息記錄" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="風險評估" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="每日更新記錄" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -912,7 +912,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-10-01</t>
+          <t>報告更新日期：2026-10-02</t>
         </is>
       </c>
     </row>
@@ -3377,7 +3377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G136"/>
+  <dimension ref="A1:G137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3399,7 +3399,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-10-01</t>
+          <t>最後更新：2026-10-02</t>
         </is>
       </c>
     </row>
@@ -8518,6 +8518,49 @@
         </is>
       </c>
     </row>
+    <row r="137">
+      <c r="A137" s="50" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B137" s="50" t="inlineStr">
+        <is>
+          <t>NT$2,510（10/1收，+30；開2,490低2,485收最高2,510，平6/22年高收盤，量縮39.7%）</t>
+        </is>
+      </c>
+      <c r="C137" s="51" t="inlineStr">
+        <is>
+          <t>+1.21%（10/1收，+30.00，領先大盤0.35pp；加權+0.86%創收盤新高）</t>
+        </is>
+      </c>
+      <c r="D137" s="50" t="inlineStr">
+        <is>
+          <t>US$459.20（10/1收，+0.66%；費半+1.59%；ADR溢價+16.50%）</t>
+        </is>
+      </c>
+      <c r="E137" s="50" t="inlineStr">
+        <is>
+          <t>20,666（10/1收，-39.7%，低於5日均量23,843張13.3%、低於9月中位數3.1%）</t>
+        </is>
+      </c>
+      <c r="F137" s="52" t="inlineStr">
+        <is>
+          <t>報告日2026-10-02(Fri)。台股資料為2026-10-01(Thu，第四季首個交易日)TWSE官方收盤；ADR、費半與美股個股為10/1正式收盤(Yahoo meta 16:00 ET)；韓股為10/1收盤(Yahoo日K，確有交易；陸媒「國軍節休市」說法判為錯誤)；期貨為TAIFEX 10/1日盤＋今晨夜盤(10/1 15:00至10/2約05:00)；匯率採台北外匯10/1收盤31.842；全市場法人金額採BFI82U官方。
+(1)⭐⭐10/1台股2330開高走高收全日最高2,510(+30、+1.21%)，平6/22的2026年最高收盤、首度收在2,495–2,510壓力區上緣(開2,490／低2,485，缺口2,480–2,485未回補)；加權+413.36點(+0.86%)收48,353.49創收盤新高，台積電領先0.35pp。⚠️量20,666張萎縮39.7%(金額NT$517.02億、57,634筆)，低於5日均量23,843張13.3%、低於9月中位數3.1%，為縮量創高。
+(2)⭐前報六項檢核：守2,475通過(9/30黑K頭部警訊解除)；回撤條件(MA10 2,452／外資賣逾5,000張)未觸發；上調條件「收≥2,510且量≥24,112張」只過價格、量能不過→依判準不上調；夜盤2,505指示開+10收+30兩端兌現(累計開6/7收4/7)；美光10/1正式收盤+3.03%收$1,097.39、僅兌現盤後約+12%的四分之一(利多出盡部分應驗)；外資連2買且集中度自5.6%回升至35.4%；P/C新週期第2日82.54%。
+(3)⭐籌碼：外資+3,090張(買14,212,490股／賣11,121,760股，連2買、2日合計3,792張，占全市場外資買超219.37億的35.4%)、投信+596(連3買)、自營+602(連12買)，三大法人官方合計+4,289張；全市場三大法人+NT$294.62億(外資+219.37／投信+58.65／自營自行+32.37／避險-15.78，BFI82U官方)。⚠️外資台指期淨空-79,554口(再擴大1,403口，空單91,927口為追蹤以來最高)，現貨買、期貨空背離重現。
+(4)⭐技術(TWSE官方序列180日自算)：RSI 61.37(超越9/23的60.97、7/01以來最高)、MACD柱+11.75(中止連3日縮小；DIF 23.91連9升／DEA 18.04)、K 82.68／D 72.49／J 103.05(重返100之上，9/23以來首度)；MA5 2,488／MA10 2,465／MA20 2,443／MA60 2,403／MA120 2,338五線多頭連6日；布林2,359–2,443–2,526、寬度6.81%。衍生品：個股期日盤收2,530(+30)、OI 25,362、基差+20，今晨夜盤收2,515(較結算-15、較現貨+5)；台指期48,685(+0.73%)、夜盤48,475(-210)；CDO近月call 317(單日+127、集中2,650–2,700)／put 110口、最大痛點2,500。
+(5)⭐美股10/1費半+200.38點(+1.59%)收12,829.00、ADR +0.66%收$459.20(溢價+16.50%、自17.17%收斂)；19檔供應鏈14漲5跌：科林+3.53%、應材+3.50%、科磊+2.77%、美光+3.03%、SK海力士+3.21%、三星+2.79%、輝達+1.09%；博通-2.15%、高通-1.06%(連4黑)、蘋果-0.81%、艾司摩爾-0.18%、英特爾-0.19%；台股聯發科+1.22%、日月光+1.00%、華邦電+0.28%。消息：美10年期殖利率盤中5.34%創2002年以來新高、收5.24%【媒體數】；9月ISM製造業PMI 54.5；美光26份長約、承諾US$320億【媒體數】；台積電德州第二園區評估延燒、董事會未拍板。BWIBBU P/E 29.09x(追蹤以來最高)／P/B 10.12x／殖利率0.88%。
+(6)立場維持「中性偏多」、不上調，首要保留改為「縮量創高」與「現貨買、期貨空」背離。次日(10/2週五)檢核：收≥2,515且量≥23,843張→上調；跌回2,495之下且量增、或跌破MA10 2,465、或外資單日賣逾5,000張→退回中性；J過100後回落風險；夜盤「持平至小幅偏弱」指示兌現；外資能否連3買、期貨空單是否續擴大。9月營收約10/10前後(官方未公告；10/9國慶補假休市【待核對】)、緘默期10/5起、Q3法說10/15。</t>
+        </is>
+      </c>
+      <c r="G137" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:G2"/>

</xml_diff>

<commit_message>
daily: 2026-10-06 日報 HTML & Excel 更新（補涵蓋 10/02 與 10/05 兩個交易日，10/05 日報漏跑）
- 10/02 收 2,500（-0.40%、量 15,792 張）外資賣超 5,913 張觸發前報退回條件→中性
- 10/05 收 2,575（+3.00%、量 26,800 張）收盤與盤中高 2,580 皆歷史新高、外資買超 9,770 張，
  前報上調條件成立→中性偏多（不再上調看多：高於布林上軌 23 元、J 101.8、外資台指期淨空 -77,004 口）
- 法人 5 日陣列前推兩格、RELATIVE/VALUATION/FX/EPS_REVISION/CONSENSUS upside/52 週高低同步更新
- 估值解讀模板的均值回歸價由寫死 NT$1,200 改為動態計算（本報 NT$1,595）
- fresh-context 驗收 12 條：10 通過、2 不通過已於本 commit 內更正（量能定性基準、均值回歸價）
- Excel 每日更新記錄第 138 列

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -912,7 +912,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-10-02</t>
+          <t>報告更新日期：2026-10-06</t>
         </is>
       </c>
     </row>
@@ -3377,7 +3377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G137"/>
+  <dimension ref="A1:G138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3399,7 +3399,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-10-02</t>
+          <t>最後更新：2026-10-06</t>
         </is>
       </c>
     </row>
@@ -8561,6 +8561,43 @@
         </is>
       </c>
     </row>
+    <row r="138">
+      <c r="A138" s="53" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B138" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,575（10/5收，+75；開2,550高2,580低2,545，收盤與盤中高皆創歷史新高）；10/2收NT$2,500（-10）</t>
+        </is>
+      </c>
+      <c r="C138" s="54" t="inlineStr">
+        <is>
+          <t>+3.00%（10/5收，+75.00，領先大盤0.45pp；加權+2.55%創收盤新高）；10/2為-0.40%（-10.00，落後大盤0.65pp）</t>
+        </is>
+      </c>
+      <c r="D138" s="53" t="inlineStr">
+        <is>
+          <t>US$485.80（10/5收，+2.75%，近兩年最高收盤；ADR溢價+19.95%）；10/2收US$472.78（+2.96%）</t>
+        </is>
+      </c>
+      <c r="E138" s="53" t="inlineStr">
+        <is>
+          <t>26,800（10/5收，+69.7%，高於5日均量24,887張7.7%；2026年182日中由大到小第138）；10/2為15,792張（2026年第9低）</t>
+        </is>
+      </c>
+      <c r="F138" s="55" t="inlineStr">
+        <is>
+          <t>報告日2026-10-06。本報涵蓋10/2與10/5兩個台股交易日，10/5之日報未產製。10/2收2,500(-0.40%)，外資賣超5,913張觸發退回中性；10/5收2,575(+3.00%)創歷史新高、量26,800張、外資買超9,770張，上調條件成立、回到中性偏多，因短線過熱不再上調。</t>
+        </is>
+      </c>
+      <c r="G138" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:G2"/>

</xml_diff>

<commit_message>
daily: 2026-10-07 日報 HTML & Excel 更新
- 涵蓋 10/06（二）單一交易日：2330 收 2,585（+10、+0.39%）收盤與盤中 2,590 皆創歷史新高，量 20,802 張；外資小賣 1,672 張、投信連 6 日、自營連 15 日買超
- NYSE TSM 收 482.30（-0.72%）、ADR 溢價 +18.59%；費半 +0.34%，S&P 500／那斯達克創新高
- 立場維持「中性偏多」：前報上調條件只過價格（量與外資未過）；新訂 10/07 檢核條件
- 修正既存問題：CASHFLOW 的 FCF 殖利率改依 STOCK 市值動態計算（原寫死 NT$49.27T 舊市值）；IR_CALENDAR 5/26、7/16 星期標記更正
- Fresh-context 驗收：12 條中 10 條通過，2 條不通過（皆既存舊問題）已於本 commit 修正

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -912,7 +912,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-10-06</t>
+          <t>報告更新日期：2026-10-07</t>
         </is>
       </c>
     </row>
@@ -3377,7 +3377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G138"/>
+  <dimension ref="A1:G139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3399,7 +3399,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-10-06</t>
+          <t>最後更新：2026-10-07</t>
         </is>
       </c>
     </row>
@@ -8598,6 +8598,43 @@
         </is>
       </c>
     </row>
+    <row r="139">
+      <c r="A139" s="50" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B139" s="50" t="inlineStr">
+        <is>
+          <t>NT$2,585（10/6收，+10；開2,575高2,590低2,565，收盤與盤中高連2日創歷史新高）；10/5收NT$2,575（+75）</t>
+        </is>
+      </c>
+      <c r="C139" s="51" t="inlineStr">
+        <is>
+          <t>+0.39%（10/6收，+10.00，領先大盤0.17pp；加權+0.22%連4日創收盤新高）；10/5為+3.00%（+75.00）</t>
+        </is>
+      </c>
+      <c r="D139" s="50" t="inlineStr">
+        <is>
+          <t>US$482.30（10/6收，-0.72%，未創新高；ADR溢價+18.59%）；10/5收US$485.80（+2.75%）</t>
+        </is>
+      </c>
+      <c r="E139" s="50" t="inlineStr">
+        <is>
+          <t>20,802（10/6收，-22.4%，低於前報門檻24,887張16.4%、低於5日均量23,669張12.1%；2026年183日中第23低）；10/5為26,800張</t>
+        </is>
+      </c>
+      <c r="F139" s="52" t="inlineStr">
+        <is>
+          <t>報告日2026-10-07。10/6收2,585(+0.39%)連2日創歷史收盤新高，但量縮至20,802張、外資賣超1,672張，前報上調看多條件只過價格，維持中性偏多；退回中性防線皆守住，收盤續高於布林上軌，過熱未解。</t>
+        </is>
+      </c>
+      <c r="G139" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:G2"/>

</xml_diff>

<commit_message>
daily: 2026-10-08 日報 HTML & Excel 更新
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -912,7 +912,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-10-07</t>
+          <t>報告更新日期：2026-10-08</t>
         </is>
       </c>
     </row>
@@ -3377,7 +3377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G139"/>
+  <dimension ref="A1:G140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3399,7 +3399,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-10-07</t>
+          <t>最後更新：2026-10-08</t>
         </is>
       </c>
     </row>
@@ -8635,6 +8635,43 @@
         </is>
       </c>
     </row>
+    <row r="140">
+      <c r="A140" s="53" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B140" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,585（10/7收，平盤0.00；開2,565高2,585低2,560，與10/6歷史最高收盤同價、未再創新高）；10/6收NT$2,585（+10）</t>
+        </is>
+      </c>
+      <c r="C140" s="56" t="inlineStr">
+        <is>
+          <t>0.00%（10/7收，平盤，相對大盤+0.03pp；加權-0.03%、連4日創收盤新高中止）；10/6為+0.39%（+10.00）</t>
+        </is>
+      </c>
+      <c r="D140" s="53" t="inlineStr">
+        <is>
+          <t>US$472.20（10/7收，-2.09%，跌幅為費半-1.15%的1.8倍；ADR溢價+16.18%、連2日收斂）；10/6收US$482.30（-0.72%）</t>
+        </is>
+      </c>
+      <c r="E140" s="53" t="inlineStr">
+        <is>
+          <t>16,941（10/7收，-18.6%，低於前報基準23,669張28.4%、低於新5日均量20,200張16.1%；2026年184日中第11低）；10/6為20,802張</t>
+        </is>
+      </c>
+      <c r="F140" s="55" t="inlineStr">
+        <is>
+          <t>報告日2026-10-08。10/7開低拉回收平盤2,585，平歷史最高收盤但未創新高，量再縮至16,941張、外資連2日小賣1,163張，上調看多三條件全部未過、退回防線守住，維持中性偏多但信心標低；ADR-2.09%、夜盤個股期2,570低於現貨，連假前偏弱。</t>
+        </is>
+      </c>
+      <c r="G140" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:G2"/>

</xml_diff>

<commit_message>
daily: 2026-10-13 日報 HTML & Excel 更新（台股 10/12 收 2,540 -0.39%、外資連 4 賣；ADR 10/12 444.35 -1.98% 連 5 跌、溢價 +11.61%；立場依既定門檻 2,545 由中性下修為中性偏空）
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -912,7 +912,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-10-12</t>
+          <t>報告更新日期：2026-10-13</t>
         </is>
       </c>
     </row>
@@ -3377,7 +3377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G141"/>
+  <dimension ref="A1:G142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3399,7 +3399,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-10-12</t>
+          <t>最後更新：2026-10-13</t>
         </is>
       </c>
     </row>
@@ -8709,6 +8709,43 @@
         </is>
       </c>
     </row>
+    <row r="142">
+      <c r="A142" s="53" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B142" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,540（10/12收，-10、-0.39%；開2,510高2,550低2,510，開低40元回補10/5缺口後拉回、紅K但跌破2,545防線5元；10/9國慶補假休市後首日）；10/8收NT$2,550（-1.35%）</t>
+        </is>
+      </c>
+      <c r="C142" s="56" t="inlineStr">
+        <is>
+          <t>-0.39%（10/12收，相對大盤-0.37pp；加權-11.48點、-0.02%收49,301.96、連3日下跌）；10/8為-1.35%</t>
+        </is>
+      </c>
+      <c r="D142" s="53" t="inlineStr">
+        <is>
+          <t>US$444.35（10/12收，-1.98%；連5日下跌、五日-8.53%、9/18以來最低；ADR溢價壓縮至+11.61%）；10/9收US$453.31（-1.02%）</t>
+        </is>
+      </c>
+      <c r="E142" s="53" t="inlineStr">
+        <is>
+          <t>23,556（10/12收，+1.8%，高於前報基準20,696張13.8%、高於新5日均量22,249張5.9%；成交筆數125,197筆；2026年186日中第153）；10/8為23,145張</t>
+        </is>
+      </c>
+      <c r="F142" s="55" t="inlineStr">
+        <is>
+          <t>報告日2026-10-13（台美皆為10/12）。10/12開低回補10/5缺口後收2,540（-0.39%），跌破防線2,545達5元，立場依約自中性下修為中性偏空；外資連4日賣超合計24,559張；台股收盤後ADR再-1.98%連5跌收444.35、溢價+11.61%，夜盤個股期2,520低於現貨20點；10/15法說會距今2天。</t>
+        </is>
+      </c>
+      <c r="G142" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:G2"/>

</xml_diff>

<commit_message>
daily: 2026-10-15 日報 HTML & Excel 更新（台股 10/14 收 2,490 平盤、外資賣超 6,752 張連 6 賣、MACD 死叉；ADR 10/14 430.00 -3.40%、費半 -4.30%、溢價 +10.76%；夜盤個股期 2,474 偏弱；立場維持看空；今日 14:00 Q3 法說）
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -334,7 +334,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -522,6 +522,9 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="12" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -912,7 +915,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-10-14</t>
+          <t>報告更新日期：2026-10-15</t>
         </is>
       </c>
     </row>
@@ -3377,7 +3380,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G143"/>
+  <dimension ref="A1:G144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3399,7 +3402,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-10-14</t>
+          <t>最後更新：2026-10-15</t>
         </is>
       </c>
     </row>
@@ -8783,6 +8786,43 @@
         </is>
       </c>
     </row>
+    <row r="144">
+      <c r="A144" s="53" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B144" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,490（10/14收，平盤0.00、0.00%；開2,505高2,535低2,490，開高後收在全日最低、黑K，盤中2,535未守住）；10/13收NT$2,490（-1.97%）</t>
+        </is>
+      </c>
+      <c r="C144" s="66" t="inlineStr">
+        <is>
+          <t>0.00%（10/14收，平盤，相對大盤-0.59pp；加權+284.52點、+0.59%收48,625.83、結束連4日下跌）；10/13為-1.97%</t>
+        </is>
+      </c>
+      <c r="D144" s="53" t="inlineStr">
+        <is>
+          <t>US$430.00（10/14收，-3.40%；9/16以來最低收盤、五日-8.94%；ADR溢價壓縮至+10.76%）；10/13收US$445.12（+0.17%）</t>
+        </is>
+      </c>
+      <c r="E144" s="53" t="inlineStr">
+        <is>
+          <t>28,112（10/14收，-31.1%；高於前報基準25,048張12.2%、高於新5日均量26,510張6.0%；成交筆數91,202筆；2026年188日中第133）；10/13為40,796張</t>
+        </is>
+      </c>
+      <c r="F144" s="55" t="inlineStr">
+        <is>
+          <t>報告日2026-10-15（台美皆為10/14）。10/14開高後收全日最低2,490（平盤），外資賣超6,752張（連6賣），立場維持看空；MACD死叉；美股CPI偏熱、費半-4.30%，ADR-3.40%收430.00、溢價+10.76%，夜盤個股期2,474；Q3法說會今日14:00。</t>
+        </is>
+      </c>
+      <c r="G144" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:G2"/>

</xml_diff>

<commit_message>
daily: 2026-10-19 日報 HTML & Excel 更新（台股 10/16 收 2,420 -0.82%、量 43,047 張、外資賣超 22,046 張連 8 賣（累計 113,109 張）、收盤貼 MA60 2,421 下 1 元、MACD 柱 -26.94、K 18.94；外資台指期淨空 -93,675 口較前日回補 3,907 口；ADR 10/16 412.61 -2.28%、費半 -3.83% 連 8 跌、溢價 +10.28%（央行 32.338→32.34）；夜盤個股期 2,384 偏弱、台指期 -1,144；Aletheia 目標價 5,000、野村 3,745；立場維持看空；fresh-context 驗收 8 項全數通過）
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="600" firstSheet="0" activeTab="6" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="封面總覽" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="財務摘要" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="營收結構分析" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="2026展望" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="股息記錄" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="風險評估" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="每日更新記錄" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="封面總覽" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="財務摘要" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="營收結構分析" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026展望" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="股息記錄" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="風險評估" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="每日更新記錄" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -915,7 +915,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-10-16</t>
+          <t>報告更新日期：2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3402,7 +3402,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G145"/>
+  <dimension ref="A1:G146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3424,7 +3424,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-10-16</t>
+          <t>最後更新：2026-10-19</t>
         </is>
       </c>
     </row>
@@ -8882,6 +8882,43 @@
         </is>
       </c>
     </row>
+    <row r="146">
+      <c r="A146" s="53" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B146" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,420（10/16收，-20、-0.82%；開2,430高2,445低2,420，開低走低收最低小黑K，2,450–2,490缺口未回補，收盤低於MA60 2,421僅1元）；10/15收NT$2,440（-2.01%）</t>
+        </is>
+      </c>
+      <c r="C146" s="56" t="inlineStr">
+        <is>
+          <t>-0.82%（10/16收，相對大盤-1.12pp；加權+141.39點、+0.30%收47,111.26，全市場成交9,938.15億）；10/15為-2.01%</t>
+        </is>
+      </c>
+      <c r="D146" s="53" t="inlineStr">
+        <is>
+          <t>US$412.61（10/16收，-2.28%；連3跌、8/24以來最低、五日-8.98%；ADR溢價收斂至+10.28%）；10/15收US$422.25（-1.80%）</t>
+        </is>
+      </c>
+      <c r="E146" s="53" t="inlineStr">
+        <is>
+          <t>43,047（10/16收，-26.4%；高於前報基準34,819張23.6%、高於新5日均量38,800張10.9%；2026年190日中第57）；10/15為58,487張</t>
+        </is>
+      </c>
+      <c r="F146" s="55" t="inlineStr">
+        <is>
+          <t>10/16法說後首日收最低2,420（-0.82%），外資賣超22,046張連8賣、低於MA60 1元，維持看空；費半-3.83%、ADR-2.28%，夜盤偏弱。</t>
+        </is>
+      </c>
+      <c r="G146" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:G2"/>

</xml_diff>